<commit_message>
fix(pr30): trim empty tails from declaration templates to fit A4
Шаблоны Form_A и Form_B имели огромные пустые хвосты в листах: Р.1.1 в Form_B
заканчивался на row 51, но имел max_row=119 — 70 пустых строк по ~12pt = 926pt
мёртвого пространства. Из-за этого общая высота листа была 1762pt — в 2 раза
больше A4 (842pt), и soffice применял scale ~47% при PDF-конвертации, что
делало текст крупнее, а штамп-зону 84pt — мельче.

После обрезки хвостов все 4 листа близки к A4:
- Титульный лист: 823pt
- Р.1.1: 836pt (было 1762pt)
- Р.2.1.1: 599pt
- Р.2.1.1 (продол.): 791pt

Padding 84pt (9pt + 75pt) сохранён в конце каждого листа для штампа ЭДО.
Координаты filler-функций остались прежними — мы не трогали верхние строки.
</commit_message>
<xml_diff>
--- a/modules/usn_declaration/data/declaration_template_2025.xlsx
+++ b/modules/usn_declaration/data/declaration_template_2025.xlsx
@@ -1675,7 +1675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN64"/>
+  <dimension ref="A1:AN62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="121" min="1" max="13"/>
@@ -4206,193 +4206,10 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="4.5" customHeight="1" s="122"/>
-    <row r="62" ht="13.5" customHeight="1" s="122">
-      <c r="A62" s="123" t="n"/>
-      <c r="B62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="E62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="F62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="G62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="H62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="I62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="J62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="K62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="L62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="M62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="N62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="O62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="P62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="Q62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="R62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="S62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="T62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="U62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="V62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="W62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="X62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="Y62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="Z62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AA62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AB62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AC62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AD62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AE62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AF62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AG62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AH62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AI62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AJ62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AK62" s="121" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN62" s="123" t="n"/>
-    </row>
-    <row r="63" ht="9" customHeight="1" s="122"/>
-    <row r="64" ht="75" customHeight="1" s="122"/>
+    <row r="61" ht="9" customHeight="1" s="122"/>
+    <row r="62" ht="75" customHeight="1" s="122"/>
+    <row r="63" ht="17.25" customHeight="1" s="122"/>
+    <row r="64" ht="17.25" customHeight="1" s="122"/>
     <row r="65" ht="17.25" customHeight="1" s="122"/>
     <row r="516" ht="17.25" customHeight="1" s="122"/>
   </sheetData>
@@ -9985,7 +9802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN123"/>
+  <dimension ref="A1:AN53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="121" min="1" max="12"/>
@@ -11458,1898 +11275,78 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="12.75" customHeight="1" s="122">
-      <c r="A52" s="173" t="n"/>
-      <c r="B52" s="173" t="n"/>
-      <c r="C52" s="173" t="n"/>
-      <c r="D52" s="173" t="n"/>
-      <c r="E52" s="173" t="n"/>
-      <c r="F52" s="173" t="n"/>
-      <c r="G52" s="173" t="n"/>
-      <c r="H52" s="173" t="n"/>
-      <c r="I52" s="173" t="n"/>
-      <c r="J52" s="173" t="n"/>
-      <c r="K52" s="173" t="n"/>
-      <c r="L52" s="173" t="n"/>
-      <c r="M52" s="173" t="n"/>
-      <c r="N52" s="173" t="n"/>
-      <c r="O52" s="173" t="n"/>
-      <c r="P52" s="173" t="n"/>
-      <c r="Q52" s="173" t="n"/>
-      <c r="R52" s="173" t="n"/>
-      <c r="S52" s="173" t="n"/>
-      <c r="T52" s="173" t="n"/>
-      <c r="U52" s="173" t="n"/>
-      <c r="V52" s="173" t="n"/>
-      <c r="W52" s="173" t="n"/>
-      <c r="X52" s="173" t="n"/>
-      <c r="Y52" s="173" t="n"/>
-    </row>
-    <row r="53" ht="12.75" customHeight="1" s="122">
-      <c r="A53" s="173" t="n"/>
-      <c r="B53" s="173" t="n"/>
-      <c r="C53" s="173" t="n"/>
-      <c r="D53" s="173" t="n"/>
-      <c r="E53" s="173" t="n"/>
-      <c r="F53" s="173" t="n"/>
-      <c r="G53" s="173" t="n"/>
-      <c r="H53" s="173" t="n"/>
-      <c r="I53" s="173" t="n"/>
-      <c r="J53" s="173" t="n"/>
-      <c r="K53" s="173" t="n"/>
-      <c r="L53" s="173" t="n"/>
-      <c r="M53" s="173" t="n"/>
-      <c r="N53" s="173" t="n"/>
-      <c r="O53" s="173" t="n"/>
-      <c r="P53" s="173" t="n"/>
-      <c r="Q53" s="173" t="n"/>
-      <c r="R53" s="173" t="n"/>
-      <c r="S53" s="173" t="n"/>
-      <c r="T53" s="173" t="n"/>
-      <c r="U53" s="173" t="n"/>
-      <c r="V53" s="173" t="n"/>
-      <c r="W53" s="173" t="n"/>
-      <c r="X53" s="173" t="n"/>
-      <c r="Y53" s="173" t="n"/>
-    </row>
-    <row r="54" ht="12.75" customHeight="1" s="122">
-      <c r="A54" s="173" t="n"/>
-      <c r="B54" s="173" t="n"/>
-      <c r="C54" s="173" t="n"/>
-      <c r="D54" s="173" t="n"/>
-      <c r="E54" s="173" t="n"/>
-      <c r="F54" s="173" t="n"/>
-      <c r="G54" s="173" t="n"/>
-      <c r="H54" s="173" t="n"/>
-      <c r="I54" s="173" t="n"/>
-      <c r="J54" s="173" t="n"/>
-      <c r="K54" s="173" t="n"/>
-      <c r="L54" s="173" t="n"/>
-      <c r="M54" s="173" t="n"/>
-      <c r="N54" s="173" t="n"/>
-      <c r="O54" s="173" t="n"/>
-      <c r="P54" s="173" t="n"/>
-      <c r="Q54" s="173" t="n"/>
-      <c r="R54" s="173" t="n"/>
-      <c r="S54" s="173" t="n"/>
-      <c r="T54" s="173" t="n"/>
-      <c r="U54" s="173" t="n"/>
-      <c r="V54" s="173" t="n"/>
-      <c r="W54" s="173" t="n"/>
-      <c r="X54" s="173" t="n"/>
-      <c r="Y54" s="173" t="n"/>
-    </row>
-    <row r="55" ht="12.75" customHeight="1" s="122">
-      <c r="A55" s="173" t="n"/>
-      <c r="B55" s="173" t="n"/>
-      <c r="C55" s="173" t="n"/>
-      <c r="D55" s="173" t="n"/>
-      <c r="E55" s="173" t="n"/>
-      <c r="F55" s="173" t="n"/>
-      <c r="G55" s="173" t="n"/>
-      <c r="H55" s="173" t="n"/>
-      <c r="I55" s="173" t="n"/>
-      <c r="J55" s="173" t="n"/>
-      <c r="K55" s="173" t="n"/>
-      <c r="L55" s="173" t="n"/>
-      <c r="M55" s="173" t="n"/>
-      <c r="N55" s="173" t="n"/>
-      <c r="O55" s="173" t="n"/>
-      <c r="P55" s="173" t="n"/>
-      <c r="Q55" s="173" t="n"/>
-      <c r="R55" s="173" t="n"/>
-      <c r="S55" s="173" t="n"/>
-      <c r="T55" s="173" t="n"/>
-      <c r="U55" s="173" t="n"/>
-      <c r="V55" s="173" t="n"/>
-      <c r="W55" s="173" t="n"/>
-      <c r="X55" s="173" t="n"/>
-      <c r="Y55" s="173" t="n"/>
-    </row>
-    <row r="56" ht="12.75" customHeight="1" s="122">
-      <c r="A56" s="173" t="n"/>
-      <c r="B56" s="173" t="n"/>
-      <c r="C56" s="173" t="n"/>
-      <c r="D56" s="173" t="n"/>
-      <c r="E56" s="173" t="n"/>
-      <c r="F56" s="173" t="n"/>
-      <c r="G56" s="173" t="n"/>
-      <c r="H56" s="173" t="n"/>
-      <c r="I56" s="173" t="n"/>
-      <c r="J56" s="173" t="n"/>
-      <c r="K56" s="173" t="n"/>
-      <c r="L56" s="173" t="n"/>
-      <c r="M56" s="173" t="n"/>
-      <c r="N56" s="173" t="n"/>
-      <c r="O56" s="173" t="n"/>
-      <c r="P56" s="173" t="n"/>
-      <c r="Q56" s="173" t="n"/>
-      <c r="R56" s="173" t="n"/>
-      <c r="S56" s="173" t="n"/>
-      <c r="T56" s="173" t="n"/>
-      <c r="U56" s="173" t="n"/>
-      <c r="V56" s="173" t="n"/>
-      <c r="W56" s="173" t="n"/>
-      <c r="X56" s="173" t="n"/>
-      <c r="Y56" s="173" t="n"/>
-    </row>
-    <row r="57" ht="12.75" customHeight="1" s="122">
-      <c r="A57" s="173" t="n"/>
-      <c r="B57" s="173" t="n"/>
-      <c r="C57" s="173" t="n"/>
-      <c r="D57" s="173" t="n"/>
-      <c r="E57" s="173" t="n"/>
-      <c r="F57" s="173" t="n"/>
-      <c r="G57" s="173" t="n"/>
-      <c r="H57" s="173" t="n"/>
-      <c r="I57" s="173" t="n"/>
-      <c r="J57" s="173" t="n"/>
-      <c r="K57" s="173" t="n"/>
-      <c r="L57" s="173" t="n"/>
-      <c r="M57" s="173" t="n"/>
-      <c r="N57" s="173" t="n"/>
-      <c r="O57" s="173" t="n"/>
-      <c r="P57" s="173" t="n"/>
-      <c r="Q57" s="173" t="n"/>
-      <c r="R57" s="173" t="n"/>
-      <c r="S57" s="173" t="n"/>
-      <c r="T57" s="173" t="n"/>
-      <c r="U57" s="173" t="n"/>
-      <c r="V57" s="173" t="n"/>
-      <c r="W57" s="173" t="n"/>
-      <c r="X57" s="173" t="n"/>
-      <c r="Y57" s="173" t="n"/>
-    </row>
-    <row r="58" ht="12.75" customHeight="1" s="122">
-      <c r="A58" s="173" t="n"/>
-      <c r="B58" s="173" t="n"/>
-      <c r="C58" s="173" t="n"/>
-      <c r="D58" s="173" t="n"/>
-      <c r="E58" s="173" t="n"/>
-      <c r="F58" s="173" t="n"/>
-      <c r="G58" s="173" t="n"/>
-      <c r="H58" s="173" t="n"/>
-      <c r="I58" s="173" t="n"/>
-      <c r="J58" s="173" t="n"/>
-      <c r="K58" s="173" t="n"/>
-      <c r="L58" s="173" t="n"/>
-      <c r="M58" s="173" t="n"/>
-      <c r="N58" s="173" t="n"/>
-      <c r="O58" s="173" t="n"/>
-      <c r="P58" s="173" t="n"/>
-      <c r="Q58" s="173" t="n"/>
-      <c r="R58" s="173" t="n"/>
-      <c r="S58" s="173" t="n"/>
-      <c r="T58" s="173" t="n"/>
-      <c r="U58" s="173" t="n"/>
-      <c r="V58" s="173" t="n"/>
-      <c r="W58" s="173" t="n"/>
-      <c r="X58" s="173" t="n"/>
-      <c r="Y58" s="173" t="n"/>
-    </row>
-    <row r="59" ht="12.75" customHeight="1" s="122">
-      <c r="A59" s="173" t="n"/>
-      <c r="B59" s="173" t="n"/>
-      <c r="C59" s="173" t="n"/>
-      <c r="D59" s="173" t="n"/>
-      <c r="E59" s="173" t="n"/>
-      <c r="F59" s="173" t="n"/>
-      <c r="G59" s="173" t="n"/>
-      <c r="H59" s="173" t="n"/>
-      <c r="I59" s="173" t="n"/>
-      <c r="J59" s="173" t="n"/>
-      <c r="K59" s="173" t="n"/>
-      <c r="L59" s="173" t="n"/>
-      <c r="M59" s="173" t="n"/>
-      <c r="N59" s="173" t="n"/>
-      <c r="O59" s="173" t="n"/>
-      <c r="P59" s="173" t="n"/>
-      <c r="Q59" s="173" t="n"/>
-      <c r="R59" s="173" t="n"/>
-      <c r="S59" s="173" t="n"/>
-      <c r="T59" s="173" t="n"/>
-      <c r="U59" s="173" t="n"/>
-      <c r="V59" s="173" t="n"/>
-      <c r="W59" s="173" t="n"/>
-      <c r="X59" s="173" t="n"/>
-      <c r="Y59" s="173" t="n"/>
-    </row>
-    <row r="60" ht="12.75" customHeight="1" s="122">
-      <c r="A60" s="173" t="n"/>
-      <c r="B60" s="173" t="n"/>
-      <c r="C60" s="173" t="n"/>
-      <c r="D60" s="173" t="n"/>
-      <c r="E60" s="173" t="n"/>
-      <c r="F60" s="173" t="n"/>
-      <c r="G60" s="173" t="n"/>
-      <c r="H60" s="173" t="n"/>
-      <c r="I60" s="173" t="n"/>
-      <c r="J60" s="173" t="n"/>
-      <c r="K60" s="173" t="n"/>
-      <c r="L60" s="173" t="n"/>
-      <c r="M60" s="173" t="n"/>
-      <c r="N60" s="173" t="n"/>
-      <c r="O60" s="173" t="n"/>
-      <c r="P60" s="173" t="n"/>
-      <c r="Q60" s="173" t="n"/>
-      <c r="R60" s="173" t="n"/>
-      <c r="S60" s="173" t="n"/>
-      <c r="T60" s="173" t="n"/>
-      <c r="U60" s="173" t="n"/>
-      <c r="V60" s="173" t="n"/>
-      <c r="W60" s="173" t="n"/>
-      <c r="X60" s="173" t="n"/>
-      <c r="Y60" s="173" t="n"/>
-    </row>
-    <row r="61" ht="12.75" customHeight="1" s="122">
-      <c r="A61" s="173" t="n"/>
-      <c r="B61" s="173" t="n"/>
-      <c r="C61" s="173" t="n"/>
-      <c r="D61" s="173" t="n"/>
-      <c r="E61" s="173" t="n"/>
-      <c r="F61" s="173" t="n"/>
-      <c r="G61" s="173" t="n"/>
-      <c r="H61" s="173" t="n"/>
-      <c r="I61" s="173" t="n"/>
-      <c r="J61" s="173" t="n"/>
-      <c r="K61" s="173" t="n"/>
-      <c r="L61" s="173" t="n"/>
-      <c r="M61" s="173" t="n"/>
-      <c r="N61" s="173" t="n"/>
-      <c r="O61" s="173" t="n"/>
-      <c r="P61" s="173" t="n"/>
-      <c r="Q61" s="173" t="n"/>
-      <c r="R61" s="173" t="n"/>
-      <c r="S61" s="173" t="n"/>
-      <c r="T61" s="173" t="n"/>
-      <c r="U61" s="173" t="n"/>
-      <c r="V61" s="173" t="n"/>
-      <c r="W61" s="173" t="n"/>
-      <c r="X61" s="173" t="n"/>
-      <c r="Y61" s="173" t="n"/>
-    </row>
-    <row r="62" ht="12.75" customHeight="1" s="122">
-      <c r="A62" s="173" t="n"/>
-      <c r="B62" s="173" t="n"/>
-      <c r="C62" s="173" t="n"/>
-      <c r="D62" s="173" t="n"/>
-      <c r="E62" s="173" t="n"/>
-      <c r="F62" s="173" t="n"/>
-      <c r="G62" s="173" t="n"/>
-      <c r="H62" s="173" t="n"/>
-      <c r="I62" s="173" t="n"/>
-      <c r="J62" s="173" t="n"/>
-      <c r="K62" s="173" t="n"/>
-      <c r="L62" s="173" t="n"/>
-      <c r="M62" s="173" t="n"/>
-      <c r="N62" s="173" t="n"/>
-      <c r="O62" s="173" t="n"/>
-      <c r="P62" s="173" t="n"/>
-      <c r="Q62" s="173" t="n"/>
-      <c r="R62" s="173" t="n"/>
-      <c r="S62" s="173" t="n"/>
-      <c r="T62" s="173" t="n"/>
-      <c r="U62" s="173" t="n"/>
-      <c r="V62" s="173" t="n"/>
-      <c r="W62" s="173" t="n"/>
-      <c r="X62" s="173" t="n"/>
-      <c r="Y62" s="173" t="n"/>
-    </row>
-    <row r="63" ht="12.75" customHeight="1" s="122">
-      <c r="A63" s="173" t="n"/>
-      <c r="B63" s="173" t="n"/>
-      <c r="C63" s="173" t="n"/>
-      <c r="D63" s="173" t="n"/>
-      <c r="E63" s="173" t="n"/>
-      <c r="F63" s="173" t="n"/>
-      <c r="G63" s="173" t="n"/>
-      <c r="H63" s="173" t="n"/>
-      <c r="I63" s="173" t="n"/>
-      <c r="J63" s="173" t="n"/>
-      <c r="K63" s="173" t="n"/>
-      <c r="L63" s="173" t="n"/>
-      <c r="M63" s="173" t="n"/>
-      <c r="N63" s="173" t="n"/>
-      <c r="O63" s="173" t="n"/>
-      <c r="P63" s="173" t="n"/>
-      <c r="Q63" s="173" t="n"/>
-      <c r="R63" s="173" t="n"/>
-      <c r="S63" s="173" t="n"/>
-      <c r="T63" s="173" t="n"/>
-      <c r="U63" s="173" t="n"/>
-      <c r="V63" s="173" t="n"/>
-      <c r="W63" s="173" t="n"/>
-      <c r="X63" s="173" t="n"/>
-      <c r="Y63" s="173" t="n"/>
-    </row>
-    <row r="64" ht="12.75" customHeight="1" s="122">
-      <c r="A64" s="173" t="n"/>
-      <c r="B64" s="173" t="n"/>
-      <c r="C64" s="173" t="n"/>
-      <c r="D64" s="173" t="n"/>
-      <c r="E64" s="173" t="n"/>
-      <c r="F64" s="173" t="n"/>
-      <c r="G64" s="173" t="n"/>
-      <c r="H64" s="173" t="n"/>
-      <c r="I64" s="173" t="n"/>
-      <c r="J64" s="173" t="n"/>
-      <c r="K64" s="173" t="n"/>
-      <c r="L64" s="173" t="n"/>
-      <c r="M64" s="173" t="n"/>
-      <c r="N64" s="173" t="n"/>
-      <c r="O64" s="173" t="n"/>
-      <c r="P64" s="173" t="n"/>
-      <c r="Q64" s="173" t="n"/>
-      <c r="R64" s="173" t="n"/>
-      <c r="S64" s="173" t="n"/>
-      <c r="T64" s="173" t="n"/>
-      <c r="U64" s="173" t="n"/>
-      <c r="V64" s="173" t="n"/>
-      <c r="W64" s="173" t="n"/>
-      <c r="X64" s="173" t="n"/>
-      <c r="Y64" s="173" t="n"/>
-    </row>
-    <row r="65" ht="12.75" customHeight="1" s="122">
-      <c r="A65" s="173" t="n"/>
-      <c r="B65" s="173" t="n"/>
-      <c r="C65" s="173" t="n"/>
-      <c r="D65" s="173" t="n"/>
-      <c r="E65" s="173" t="n"/>
-      <c r="F65" s="173" t="n"/>
-      <c r="G65" s="173" t="n"/>
-      <c r="H65" s="173" t="n"/>
-      <c r="I65" s="173" t="n"/>
-      <c r="J65" s="173" t="n"/>
-      <c r="K65" s="173" t="n"/>
-      <c r="L65" s="173" t="n"/>
-      <c r="M65" s="173" t="n"/>
-      <c r="N65" s="173" t="n"/>
-      <c r="O65" s="173" t="n"/>
-      <c r="P65" s="173" t="n"/>
-      <c r="Q65" s="173" t="n"/>
-      <c r="R65" s="173" t="n"/>
-      <c r="S65" s="173" t="n"/>
-      <c r="T65" s="173" t="n"/>
-      <c r="U65" s="173" t="n"/>
-      <c r="V65" s="173" t="n"/>
-      <c r="W65" s="173" t="n"/>
-      <c r="X65" s="173" t="n"/>
-      <c r="Y65" s="173" t="n"/>
-    </row>
-    <row r="66" ht="12.75" customHeight="1" s="122">
-      <c r="A66" s="173" t="n"/>
-      <c r="B66" s="173" t="n"/>
-      <c r="C66" s="173" t="n"/>
-      <c r="D66" s="173" t="n"/>
-      <c r="E66" s="173" t="n"/>
-      <c r="F66" s="173" t="n"/>
-      <c r="G66" s="173" t="n"/>
-      <c r="H66" s="173" t="n"/>
-      <c r="I66" s="173" t="n"/>
-      <c r="J66" s="173" t="n"/>
-      <c r="K66" s="173" t="n"/>
-      <c r="L66" s="173" t="n"/>
-      <c r="M66" s="173" t="n"/>
-      <c r="N66" s="173" t="n"/>
-      <c r="O66" s="173" t="n"/>
-      <c r="P66" s="173" t="n"/>
-      <c r="Q66" s="173" t="n"/>
-      <c r="R66" s="173" t="n"/>
-      <c r="S66" s="173" t="n"/>
-      <c r="T66" s="173" t="n"/>
-      <c r="U66" s="173" t="n"/>
-      <c r="V66" s="173" t="n"/>
-      <c r="W66" s="173" t="n"/>
-      <c r="X66" s="173" t="n"/>
-      <c r="Y66" s="173" t="n"/>
-    </row>
-    <row r="67" ht="12.75" customHeight="1" s="122">
-      <c r="A67" s="173" t="n"/>
-      <c r="B67" s="173" t="n"/>
-      <c r="C67" s="173" t="n"/>
-      <c r="D67" s="173" t="n"/>
-      <c r="E67" s="173" t="n"/>
-      <c r="F67" s="173" t="n"/>
-      <c r="G67" s="173" t="n"/>
-      <c r="H67" s="173" t="n"/>
-      <c r="I67" s="173" t="n"/>
-      <c r="J67" s="173" t="n"/>
-      <c r="K67" s="173" t="n"/>
-      <c r="L67" s="173" t="n"/>
-      <c r="M67" s="173" t="n"/>
-      <c r="N67" s="173" t="n"/>
-      <c r="O67" s="173" t="n"/>
-      <c r="P67" s="173" t="n"/>
-      <c r="Q67" s="173" t="n"/>
-      <c r="R67" s="173" t="n"/>
-      <c r="S67" s="173" t="n"/>
-      <c r="T67" s="173" t="n"/>
-      <c r="U67" s="173" t="n"/>
-      <c r="V67" s="173" t="n"/>
-      <c r="W67" s="173" t="n"/>
-      <c r="X67" s="173" t="n"/>
-      <c r="Y67" s="173" t="n"/>
-    </row>
-    <row r="68" ht="12.75" customHeight="1" s="122">
-      <c r="A68" s="173" t="n"/>
-      <c r="B68" s="173" t="n"/>
-      <c r="C68" s="173" t="n"/>
-      <c r="D68" s="173" t="n"/>
-      <c r="E68" s="173" t="n"/>
-      <c r="F68" s="173" t="n"/>
-      <c r="G68" s="173" t="n"/>
-      <c r="H68" s="173" t="n"/>
-      <c r="I68" s="173" t="n"/>
-      <c r="J68" s="173" t="n"/>
-      <c r="K68" s="173" t="n"/>
-      <c r="L68" s="173" t="n"/>
-      <c r="M68" s="173" t="n"/>
-      <c r="N68" s="173" t="n"/>
-      <c r="O68" s="173" t="n"/>
-      <c r="P68" s="173" t="n"/>
-      <c r="Q68" s="173" t="n"/>
-      <c r="R68" s="173" t="n"/>
-      <c r="S68" s="173" t="n"/>
-      <c r="T68" s="173" t="n"/>
-      <c r="U68" s="173" t="n"/>
-      <c r="V68" s="173" t="n"/>
-      <c r="W68" s="173" t="n"/>
-      <c r="X68" s="173" t="n"/>
-      <c r="Y68" s="173" t="n"/>
-    </row>
-    <row r="69" ht="12.75" customHeight="1" s="122">
-      <c r="A69" s="173" t="n"/>
-      <c r="B69" s="173" t="n"/>
-      <c r="C69" s="173" t="n"/>
-      <c r="D69" s="173" t="n"/>
-      <c r="E69" s="173" t="n"/>
-      <c r="F69" s="173" t="n"/>
-      <c r="G69" s="173" t="n"/>
-      <c r="H69" s="173" t="n"/>
-      <c r="I69" s="173" t="n"/>
-      <c r="J69" s="173" t="n"/>
-      <c r="K69" s="173" t="n"/>
-      <c r="L69" s="173" t="n"/>
-      <c r="M69" s="173" t="n"/>
-      <c r="N69" s="173" t="n"/>
-      <c r="O69" s="173" t="n"/>
-      <c r="P69" s="173" t="n"/>
-      <c r="Q69" s="173" t="n"/>
-      <c r="R69" s="173" t="n"/>
-      <c r="S69" s="173" t="n"/>
-      <c r="T69" s="173" t="n"/>
-      <c r="U69" s="173" t="n"/>
-      <c r="V69" s="173" t="n"/>
-      <c r="W69" s="173" t="n"/>
-      <c r="X69" s="173" t="n"/>
-      <c r="Y69" s="173" t="n"/>
-    </row>
-    <row r="70" ht="12.75" customHeight="1" s="122">
-      <c r="A70" s="173" t="n"/>
-      <c r="B70" s="173" t="n"/>
-      <c r="C70" s="173" t="n"/>
-      <c r="D70" s="173" t="n"/>
-      <c r="E70" s="173" t="n"/>
-      <c r="F70" s="173" t="n"/>
-      <c r="G70" s="173" t="n"/>
-      <c r="H70" s="173" t="n"/>
-      <c r="I70" s="173" t="n"/>
-      <c r="J70" s="173" t="n"/>
-      <c r="K70" s="173" t="n"/>
-      <c r="L70" s="173" t="n"/>
-      <c r="M70" s="173" t="n"/>
-      <c r="N70" s="173" t="n"/>
-      <c r="O70" s="173" t="n"/>
-      <c r="P70" s="173" t="n"/>
-      <c r="Q70" s="173" t="n"/>
-      <c r="R70" s="173" t="n"/>
-      <c r="S70" s="173" t="n"/>
-      <c r="T70" s="173" t="n"/>
-      <c r="U70" s="173" t="n"/>
-      <c r="V70" s="173" t="n"/>
-      <c r="W70" s="173" t="n"/>
-      <c r="X70" s="173" t="n"/>
-      <c r="Y70" s="173" t="n"/>
-    </row>
-    <row r="71" ht="12.75" customHeight="1" s="122">
-      <c r="A71" s="173" t="n"/>
-      <c r="B71" s="173" t="n"/>
-      <c r="C71" s="173" t="n"/>
-      <c r="D71" s="173" t="n"/>
-      <c r="E71" s="173" t="n"/>
-      <c r="F71" s="173" t="n"/>
-      <c r="G71" s="173" t="n"/>
-      <c r="H71" s="173" t="n"/>
-      <c r="I71" s="173" t="n"/>
-      <c r="J71" s="173" t="n"/>
-      <c r="K71" s="173" t="n"/>
-      <c r="L71" s="173" t="n"/>
-      <c r="M71" s="173" t="n"/>
-      <c r="N71" s="173" t="n"/>
-      <c r="O71" s="173" t="n"/>
-      <c r="P71" s="173" t="n"/>
-      <c r="Q71" s="173" t="n"/>
-      <c r="R71" s="173" t="n"/>
-      <c r="S71" s="173" t="n"/>
-      <c r="T71" s="173" t="n"/>
-      <c r="U71" s="173" t="n"/>
-      <c r="V71" s="173" t="n"/>
-      <c r="W71" s="173" t="n"/>
-      <c r="X71" s="173" t="n"/>
-      <c r="Y71" s="173" t="n"/>
-    </row>
-    <row r="72" ht="12.75" customHeight="1" s="122">
-      <c r="A72" s="173" t="n"/>
-      <c r="B72" s="173" t="n"/>
-      <c r="C72" s="173" t="n"/>
-      <c r="D72" s="173" t="n"/>
-      <c r="E72" s="173" t="n"/>
-      <c r="F72" s="173" t="n"/>
-      <c r="G72" s="173" t="n"/>
-      <c r="H72" s="173" t="n"/>
-      <c r="I72" s="173" t="n"/>
-      <c r="J72" s="173" t="n"/>
-      <c r="K72" s="173" t="n"/>
-      <c r="L72" s="173" t="n"/>
-      <c r="M72" s="173" t="n"/>
-      <c r="N72" s="173" t="n"/>
-      <c r="O72" s="173" t="n"/>
-      <c r="P72" s="173" t="n"/>
-      <c r="Q72" s="173" t="n"/>
-      <c r="R72" s="173" t="n"/>
-      <c r="S72" s="173" t="n"/>
-      <c r="T72" s="173" t="n"/>
-      <c r="U72" s="173" t="n"/>
-      <c r="V72" s="173" t="n"/>
-      <c r="W72" s="173" t="n"/>
-      <c r="X72" s="173" t="n"/>
-      <c r="Y72" s="173" t="n"/>
-    </row>
-    <row r="73" ht="12.75" customHeight="1" s="122">
-      <c r="A73" s="173" t="n"/>
-      <c r="B73" s="173" t="n"/>
-      <c r="C73" s="173" t="n"/>
-      <c r="D73" s="173" t="n"/>
-      <c r="E73" s="173" t="n"/>
-      <c r="F73" s="173" t="n"/>
-      <c r="G73" s="173" t="n"/>
-      <c r="H73" s="173" t="n"/>
-      <c r="I73" s="173" t="n"/>
-      <c r="J73" s="173" t="n"/>
-      <c r="K73" s="173" t="n"/>
-      <c r="L73" s="173" t="n"/>
-      <c r="M73" s="173" t="n"/>
-      <c r="N73" s="173" t="n"/>
-      <c r="O73" s="173" t="n"/>
-      <c r="P73" s="173" t="n"/>
-      <c r="Q73" s="173" t="n"/>
-      <c r="R73" s="173" t="n"/>
-      <c r="S73" s="173" t="n"/>
-      <c r="T73" s="173" t="n"/>
-      <c r="U73" s="173" t="n"/>
-      <c r="V73" s="173" t="n"/>
-      <c r="W73" s="173" t="n"/>
-      <c r="X73" s="173" t="n"/>
-      <c r="Y73" s="173" t="n"/>
-    </row>
-    <row r="74" ht="12.75" customHeight="1" s="122">
-      <c r="A74" s="173" t="n"/>
-      <c r="B74" s="173" t="n"/>
-      <c r="C74" s="173" t="n"/>
-      <c r="D74" s="173" t="n"/>
-      <c r="E74" s="173" t="n"/>
-      <c r="F74" s="173" t="n"/>
-      <c r="G74" s="173" t="n"/>
-      <c r="H74" s="173" t="n"/>
-      <c r="I74" s="173" t="n"/>
-      <c r="J74" s="173" t="n"/>
-      <c r="K74" s="173" t="n"/>
-      <c r="L74" s="173" t="n"/>
-      <c r="M74" s="173" t="n"/>
-      <c r="N74" s="173" t="n"/>
-      <c r="O74" s="173" t="n"/>
-      <c r="P74" s="173" t="n"/>
-      <c r="Q74" s="173" t="n"/>
-      <c r="R74" s="173" t="n"/>
-      <c r="S74" s="173" t="n"/>
-      <c r="T74" s="173" t="n"/>
-      <c r="U74" s="173" t="n"/>
-      <c r="V74" s="173" t="n"/>
-      <c r="W74" s="173" t="n"/>
-      <c r="X74" s="173" t="n"/>
-      <c r="Y74" s="173" t="n"/>
-    </row>
-    <row r="75" ht="12.75" customHeight="1" s="122">
-      <c r="A75" s="173" t="n"/>
-      <c r="B75" s="173" t="n"/>
-      <c r="C75" s="173" t="n"/>
-      <c r="D75" s="173" t="n"/>
-      <c r="E75" s="173" t="n"/>
-      <c r="F75" s="173" t="n"/>
-      <c r="G75" s="173" t="n"/>
-      <c r="H75" s="173" t="n"/>
-      <c r="I75" s="173" t="n"/>
-      <c r="J75" s="173" t="n"/>
-      <c r="K75" s="173" t="n"/>
-      <c r="L75" s="173" t="n"/>
-      <c r="M75" s="173" t="n"/>
-      <c r="N75" s="173" t="n"/>
-      <c r="O75" s="173" t="n"/>
-      <c r="P75" s="173" t="n"/>
-      <c r="Q75" s="173" t="n"/>
-      <c r="R75" s="173" t="n"/>
-      <c r="S75" s="173" t="n"/>
-      <c r="T75" s="173" t="n"/>
-      <c r="U75" s="173" t="n"/>
-      <c r="V75" s="173" t="n"/>
-      <c r="W75" s="173" t="n"/>
-      <c r="X75" s="173" t="n"/>
-      <c r="Y75" s="173" t="n"/>
-    </row>
-    <row r="76" ht="12.75" customHeight="1" s="122">
-      <c r="A76" s="173" t="n"/>
-      <c r="B76" s="173" t="n"/>
-      <c r="C76" s="173" t="n"/>
-      <c r="D76" s="173" t="n"/>
-      <c r="E76" s="173" t="n"/>
-      <c r="F76" s="173" t="n"/>
-      <c r="G76" s="173" t="n"/>
-      <c r="H76" s="173" t="n"/>
-      <c r="I76" s="173" t="n"/>
-      <c r="J76" s="173" t="n"/>
-      <c r="K76" s="173" t="n"/>
-      <c r="L76" s="173" t="n"/>
-      <c r="M76" s="173" t="n"/>
-      <c r="N76" s="173" t="n"/>
-      <c r="O76" s="173" t="n"/>
-      <c r="P76" s="173" t="n"/>
-      <c r="Q76" s="173" t="n"/>
-      <c r="R76" s="173" t="n"/>
-      <c r="S76" s="173" t="n"/>
-      <c r="T76" s="173" t="n"/>
-      <c r="U76" s="173" t="n"/>
-      <c r="V76" s="173" t="n"/>
-      <c r="W76" s="173" t="n"/>
-      <c r="X76" s="173" t="n"/>
-      <c r="Y76" s="173" t="n"/>
-    </row>
-    <row r="77" ht="12.75" customHeight="1" s="122">
-      <c r="A77" s="173" t="n"/>
-      <c r="B77" s="173" t="n"/>
-      <c r="C77" s="173" t="n"/>
-      <c r="D77" s="173" t="n"/>
-      <c r="E77" s="173" t="n"/>
-      <c r="F77" s="173" t="n"/>
-      <c r="G77" s="173" t="n"/>
-      <c r="H77" s="173" t="n"/>
-      <c r="I77" s="173" t="n"/>
-      <c r="J77" s="173" t="n"/>
-      <c r="K77" s="173" t="n"/>
-      <c r="L77" s="173" t="n"/>
-      <c r="M77" s="173" t="n"/>
-      <c r="N77" s="173" t="n"/>
-      <c r="O77" s="173" t="n"/>
-      <c r="P77" s="173" t="n"/>
-      <c r="Q77" s="173" t="n"/>
-      <c r="R77" s="173" t="n"/>
-      <c r="S77" s="173" t="n"/>
-      <c r="T77" s="173" t="n"/>
-      <c r="U77" s="173" t="n"/>
-      <c r="V77" s="173" t="n"/>
-      <c r="W77" s="173" t="n"/>
-      <c r="X77" s="173" t="n"/>
-      <c r="Y77" s="173" t="n"/>
-    </row>
-    <row r="78" ht="12.75" customHeight="1" s="122">
-      <c r="A78" s="173" t="n"/>
-      <c r="B78" s="173" t="n"/>
-      <c r="C78" s="173" t="n"/>
-      <c r="D78" s="173" t="n"/>
-      <c r="E78" s="173" t="n"/>
-      <c r="F78" s="173" t="n"/>
-      <c r="G78" s="173" t="n"/>
-      <c r="H78" s="173" t="n"/>
-      <c r="I78" s="173" t="n"/>
-      <c r="J78" s="173" t="n"/>
-      <c r="K78" s="173" t="n"/>
-      <c r="L78" s="173" t="n"/>
-      <c r="M78" s="173" t="n"/>
-      <c r="N78" s="173" t="n"/>
-      <c r="O78" s="173" t="n"/>
-      <c r="P78" s="173" t="n"/>
-      <c r="Q78" s="173" t="n"/>
-      <c r="R78" s="173" t="n"/>
-      <c r="S78" s="173" t="n"/>
-      <c r="T78" s="173" t="n"/>
-      <c r="U78" s="173" t="n"/>
-      <c r="V78" s="173" t="n"/>
-      <c r="W78" s="173" t="n"/>
-      <c r="X78" s="173" t="n"/>
-      <c r="Y78" s="173" t="n"/>
-    </row>
-    <row r="79" ht="12.75" customHeight="1" s="122">
-      <c r="A79" s="173" t="n"/>
-      <c r="B79" s="173" t="n"/>
-      <c r="C79" s="173" t="n"/>
-      <c r="D79" s="173" t="n"/>
-      <c r="E79" s="173" t="n"/>
-      <c r="F79" s="173" t="n"/>
-      <c r="G79" s="173" t="n"/>
-      <c r="H79" s="173" t="n"/>
-      <c r="I79" s="173" t="n"/>
-      <c r="J79" s="173" t="n"/>
-      <c r="K79" s="173" t="n"/>
-      <c r="L79" s="173" t="n"/>
-      <c r="M79" s="173" t="n"/>
-      <c r="N79" s="173" t="n"/>
-      <c r="O79" s="173" t="n"/>
-      <c r="P79" s="173" t="n"/>
-      <c r="Q79" s="173" t="n"/>
-      <c r="R79" s="173" t="n"/>
-      <c r="S79" s="173" t="n"/>
-      <c r="T79" s="173" t="n"/>
-      <c r="U79" s="173" t="n"/>
-      <c r="V79" s="173" t="n"/>
-      <c r="W79" s="173" t="n"/>
-      <c r="X79" s="173" t="n"/>
-      <c r="Y79" s="173" t="n"/>
-    </row>
-    <row r="80" ht="12.75" customHeight="1" s="122">
-      <c r="A80" s="173" t="n"/>
-      <c r="B80" s="173" t="n"/>
-      <c r="C80" s="173" t="n"/>
-      <c r="D80" s="173" t="n"/>
-      <c r="E80" s="173" t="n"/>
-      <c r="F80" s="173" t="n"/>
-      <c r="G80" s="173" t="n"/>
-      <c r="H80" s="173" t="n"/>
-      <c r="I80" s="173" t="n"/>
-      <c r="J80" s="173" t="n"/>
-      <c r="K80" s="173" t="n"/>
-      <c r="L80" s="173" t="n"/>
-      <c r="M80" s="173" t="n"/>
-      <c r="N80" s="173" t="n"/>
-      <c r="O80" s="173" t="n"/>
-      <c r="P80" s="173" t="n"/>
-      <c r="Q80" s="173" t="n"/>
-      <c r="R80" s="173" t="n"/>
-      <c r="S80" s="173" t="n"/>
-      <c r="T80" s="173" t="n"/>
-      <c r="U80" s="173" t="n"/>
-      <c r="V80" s="173" t="n"/>
-      <c r="W80" s="173" t="n"/>
-      <c r="X80" s="173" t="n"/>
-      <c r="Y80" s="173" t="n"/>
-    </row>
-    <row r="81" ht="12.75" customHeight="1" s="122">
-      <c r="A81" s="173" t="n"/>
-      <c r="B81" s="173" t="n"/>
-      <c r="C81" s="173" t="n"/>
-      <c r="D81" s="173" t="n"/>
-      <c r="E81" s="173" t="n"/>
-      <c r="F81" s="173" t="n"/>
-      <c r="G81" s="173" t="n"/>
-      <c r="H81" s="173" t="n"/>
-      <c r="I81" s="173" t="n"/>
-      <c r="J81" s="173" t="n"/>
-      <c r="K81" s="173" t="n"/>
-      <c r="L81" s="173" t="n"/>
-      <c r="M81" s="173" t="n"/>
-      <c r="N81" s="173" t="n"/>
-      <c r="O81" s="173" t="n"/>
-      <c r="P81" s="173" t="n"/>
-      <c r="Q81" s="173" t="n"/>
-      <c r="R81" s="173" t="n"/>
-      <c r="S81" s="173" t="n"/>
-      <c r="T81" s="173" t="n"/>
-      <c r="U81" s="173" t="n"/>
-      <c r="V81" s="173" t="n"/>
-      <c r="W81" s="173" t="n"/>
-      <c r="X81" s="173" t="n"/>
-      <c r="Y81" s="173" t="n"/>
-    </row>
-    <row r="82" ht="12.75" customHeight="1" s="122">
-      <c r="A82" s="173" t="n"/>
-      <c r="B82" s="173" t="n"/>
-      <c r="C82" s="173" t="n"/>
-      <c r="D82" s="173" t="n"/>
-      <c r="E82" s="173" t="n"/>
-      <c r="F82" s="173" t="n"/>
-      <c r="G82" s="173" t="n"/>
-      <c r="H82" s="173" t="n"/>
-      <c r="I82" s="173" t="n"/>
-      <c r="J82" s="173" t="n"/>
-      <c r="K82" s="173" t="n"/>
-      <c r="L82" s="173" t="n"/>
-      <c r="M82" s="173" t="n"/>
-      <c r="N82" s="173" t="n"/>
-      <c r="O82" s="173" t="n"/>
-      <c r="P82" s="173" t="n"/>
-      <c r="Q82" s="173" t="n"/>
-      <c r="R82" s="173" t="n"/>
-      <c r="S82" s="173" t="n"/>
-      <c r="T82" s="173" t="n"/>
-      <c r="U82" s="173" t="n"/>
-      <c r="V82" s="173" t="n"/>
-      <c r="W82" s="173" t="n"/>
-      <c r="X82" s="173" t="n"/>
-      <c r="Y82" s="173" t="n"/>
-    </row>
-    <row r="83" ht="12.75" customHeight="1" s="122">
-      <c r="A83" s="173" t="n"/>
-      <c r="B83" s="173" t="n"/>
-      <c r="C83" s="173" t="n"/>
-      <c r="D83" s="173" t="n"/>
-      <c r="E83" s="173" t="n"/>
-      <c r="F83" s="173" t="n"/>
-      <c r="G83" s="173" t="n"/>
-      <c r="H83" s="173" t="n"/>
-      <c r="I83" s="173" t="n"/>
-      <c r="J83" s="173" t="n"/>
-      <c r="K83" s="173" t="n"/>
-      <c r="L83" s="173" t="n"/>
-      <c r="M83" s="173" t="n"/>
-      <c r="N83" s="173" t="n"/>
-      <c r="O83" s="173" t="n"/>
-      <c r="P83" s="173" t="n"/>
-      <c r="Q83" s="173" t="n"/>
-      <c r="R83" s="173" t="n"/>
-      <c r="S83" s="173" t="n"/>
-      <c r="T83" s="173" t="n"/>
-      <c r="U83" s="173" t="n"/>
-      <c r="V83" s="173" t="n"/>
-      <c r="W83" s="173" t="n"/>
-      <c r="X83" s="173" t="n"/>
-      <c r="Y83" s="173" t="n"/>
-    </row>
-    <row r="84" ht="12.75" customHeight="1" s="122">
-      <c r="A84" s="173" t="n"/>
-      <c r="B84" s="173" t="n"/>
-      <c r="C84" s="173" t="n"/>
-      <c r="D84" s="173" t="n"/>
-      <c r="E84" s="173" t="n"/>
-      <c r="F84" s="173" t="n"/>
-      <c r="G84" s="173" t="n"/>
-      <c r="H84" s="173" t="n"/>
-      <c r="I84" s="173" t="n"/>
-      <c r="J84" s="173" t="n"/>
-      <c r="K84" s="173" t="n"/>
-      <c r="L84" s="173" t="n"/>
-      <c r="M84" s="173" t="n"/>
-      <c r="N84" s="173" t="n"/>
-      <c r="O84" s="173" t="n"/>
-      <c r="P84" s="173" t="n"/>
-      <c r="Q84" s="173" t="n"/>
-      <c r="R84" s="173" t="n"/>
-      <c r="S84" s="173" t="n"/>
-      <c r="T84" s="173" t="n"/>
-      <c r="U84" s="173" t="n"/>
-      <c r="V84" s="173" t="n"/>
-      <c r="W84" s="173" t="n"/>
-      <c r="X84" s="173" t="n"/>
-      <c r="Y84" s="173" t="n"/>
-    </row>
-    <row r="85" ht="12.75" customHeight="1" s="122">
-      <c r="A85" s="173" t="n"/>
-      <c r="B85" s="173" t="n"/>
-      <c r="C85" s="173" t="n"/>
-      <c r="D85" s="173" t="n"/>
-      <c r="E85" s="173" t="n"/>
-      <c r="F85" s="173" t="n"/>
-      <c r="G85" s="173" t="n"/>
-      <c r="H85" s="173" t="n"/>
-      <c r="I85" s="173" t="n"/>
-      <c r="J85" s="173" t="n"/>
-      <c r="K85" s="173" t="n"/>
-      <c r="L85" s="173" t="n"/>
-      <c r="M85" s="173" t="n"/>
-      <c r="N85" s="173" t="n"/>
-      <c r="O85" s="173" t="n"/>
-      <c r="P85" s="173" t="n"/>
-      <c r="Q85" s="173" t="n"/>
-      <c r="R85" s="173" t="n"/>
-      <c r="S85" s="173" t="n"/>
-      <c r="T85" s="173" t="n"/>
-      <c r="U85" s="173" t="n"/>
-      <c r="V85" s="173" t="n"/>
-      <c r="W85" s="173" t="n"/>
-      <c r="X85" s="173" t="n"/>
-      <c r="Y85" s="173" t="n"/>
-    </row>
-    <row r="86" ht="12.75" customHeight="1" s="122">
-      <c r="A86" s="173" t="n"/>
-      <c r="B86" s="173" t="n"/>
-      <c r="C86" s="173" t="n"/>
-      <c r="D86" s="173" t="n"/>
-      <c r="E86" s="173" t="n"/>
-      <c r="F86" s="173" t="n"/>
-      <c r="G86" s="173" t="n"/>
-      <c r="H86" s="173" t="n"/>
-      <c r="I86" s="173" t="n"/>
-      <c r="J86" s="173" t="n"/>
-      <c r="K86" s="173" t="n"/>
-      <c r="L86" s="173" t="n"/>
-      <c r="M86" s="173" t="n"/>
-      <c r="N86" s="173" t="n"/>
-      <c r="O86" s="173" t="n"/>
-      <c r="P86" s="173" t="n"/>
-      <c r="Q86" s="173" t="n"/>
-      <c r="R86" s="173" t="n"/>
-      <c r="S86" s="173" t="n"/>
-      <c r="T86" s="173" t="n"/>
-      <c r="U86" s="173" t="n"/>
-      <c r="V86" s="173" t="n"/>
-      <c r="W86" s="173" t="n"/>
-      <c r="X86" s="173" t="n"/>
-      <c r="Y86" s="173" t="n"/>
-    </row>
-    <row r="87" ht="12.75" customHeight="1" s="122">
-      <c r="A87" s="173" t="n"/>
-      <c r="B87" s="173" t="n"/>
-      <c r="C87" s="173" t="n"/>
-      <c r="D87" s="173" t="n"/>
-      <c r="E87" s="173" t="n"/>
-      <c r="F87" s="173" t="n"/>
-      <c r="G87" s="173" t="n"/>
-      <c r="H87" s="173" t="n"/>
-      <c r="I87" s="173" t="n"/>
-      <c r="J87" s="173" t="n"/>
-      <c r="K87" s="173" t="n"/>
-      <c r="L87" s="173" t="n"/>
-      <c r="M87" s="173" t="n"/>
-      <c r="N87" s="173" t="n"/>
-      <c r="O87" s="173" t="n"/>
-      <c r="P87" s="173" t="n"/>
-      <c r="Q87" s="173" t="n"/>
-      <c r="R87" s="173" t="n"/>
-      <c r="S87" s="173" t="n"/>
-      <c r="T87" s="173" t="n"/>
-      <c r="U87" s="173" t="n"/>
-      <c r="V87" s="173" t="n"/>
-      <c r="W87" s="173" t="n"/>
-      <c r="X87" s="173" t="n"/>
-      <c r="Y87" s="173" t="n"/>
-    </row>
-    <row r="88" ht="12.75" customHeight="1" s="122">
-      <c r="A88" s="173" t="n"/>
-      <c r="B88" s="173" t="n"/>
-      <c r="C88" s="173" t="n"/>
-      <c r="D88" s="173" t="n"/>
-      <c r="E88" s="173" t="n"/>
-      <c r="F88" s="173" t="n"/>
-      <c r="G88" s="173" t="n"/>
-      <c r="H88" s="173" t="n"/>
-      <c r="I88" s="173" t="n"/>
-      <c r="J88" s="173" t="n"/>
-      <c r="K88" s="173" t="n"/>
-      <c r="L88" s="173" t="n"/>
-      <c r="M88" s="173" t="n"/>
-      <c r="N88" s="173" t="n"/>
-      <c r="O88" s="173" t="n"/>
-      <c r="P88" s="173" t="n"/>
-      <c r="Q88" s="173" t="n"/>
-      <c r="R88" s="173" t="n"/>
-      <c r="S88" s="173" t="n"/>
-      <c r="T88" s="173" t="n"/>
-      <c r="U88" s="173" t="n"/>
-      <c r="V88" s="173" t="n"/>
-      <c r="W88" s="173" t="n"/>
-      <c r="X88" s="173" t="n"/>
-      <c r="Y88" s="173" t="n"/>
-    </row>
-    <row r="89" ht="12.75" customHeight="1" s="122">
-      <c r="A89" s="173" t="n"/>
-      <c r="B89" s="173" t="n"/>
-      <c r="C89" s="173" t="n"/>
-      <c r="D89" s="173" t="n"/>
-      <c r="E89" s="173" t="n"/>
-      <c r="F89" s="173" t="n"/>
-      <c r="G89" s="173" t="n"/>
-      <c r="H89" s="173" t="n"/>
-      <c r="I89" s="173" t="n"/>
-      <c r="J89" s="173" t="n"/>
-      <c r="K89" s="173" t="n"/>
-      <c r="L89" s="173" t="n"/>
-      <c r="M89" s="173" t="n"/>
-      <c r="N89" s="173" t="n"/>
-      <c r="O89" s="173" t="n"/>
-      <c r="P89" s="173" t="n"/>
-      <c r="Q89" s="173" t="n"/>
-      <c r="R89" s="173" t="n"/>
-      <c r="S89" s="173" t="n"/>
-      <c r="T89" s="173" t="n"/>
-      <c r="U89" s="173" t="n"/>
-      <c r="V89" s="173" t="n"/>
-      <c r="W89" s="173" t="n"/>
-      <c r="X89" s="173" t="n"/>
-      <c r="Y89" s="173" t="n"/>
-    </row>
-    <row r="90" ht="12.75" customHeight="1" s="122">
-      <c r="A90" s="173" t="n"/>
-      <c r="B90" s="173" t="n"/>
-      <c r="C90" s="173" t="n"/>
-      <c r="D90" s="173" t="n"/>
-      <c r="E90" s="173" t="n"/>
-      <c r="F90" s="173" t="n"/>
-      <c r="G90" s="173" t="n"/>
-      <c r="H90" s="173" t="n"/>
-      <c r="I90" s="173" t="n"/>
-      <c r="J90" s="173" t="n"/>
-      <c r="K90" s="173" t="n"/>
-      <c r="L90" s="173" t="n"/>
-      <c r="M90" s="173" t="n"/>
-      <c r="N90" s="173" t="n"/>
-      <c r="O90" s="173" t="n"/>
-      <c r="P90" s="173" t="n"/>
-      <c r="Q90" s="173" t="n"/>
-      <c r="R90" s="173" t="n"/>
-      <c r="S90" s="173" t="n"/>
-      <c r="T90" s="173" t="n"/>
-      <c r="U90" s="173" t="n"/>
-      <c r="V90" s="173" t="n"/>
-      <c r="W90" s="173" t="n"/>
-      <c r="X90" s="173" t="n"/>
-      <c r="Y90" s="173" t="n"/>
-    </row>
-    <row r="91" ht="12.75" customHeight="1" s="122">
-      <c r="A91" s="173" t="n"/>
-      <c r="B91" s="173" t="n"/>
-      <c r="C91" s="173" t="n"/>
-      <c r="D91" s="173" t="n"/>
-      <c r="E91" s="173" t="n"/>
-      <c r="F91" s="173" t="n"/>
-      <c r="G91" s="173" t="n"/>
-      <c r="H91" s="173" t="n"/>
-      <c r="I91" s="173" t="n"/>
-      <c r="J91" s="173" t="n"/>
-      <c r="K91" s="173" t="n"/>
-      <c r="L91" s="173" t="n"/>
-      <c r="M91" s="173" t="n"/>
-      <c r="N91" s="173" t="n"/>
-      <c r="O91" s="173" t="n"/>
-      <c r="P91" s="173" t="n"/>
-      <c r="Q91" s="173" t="n"/>
-      <c r="R91" s="173" t="n"/>
-      <c r="S91" s="173" t="n"/>
-      <c r="T91" s="173" t="n"/>
-      <c r="U91" s="173" t="n"/>
-      <c r="V91" s="173" t="n"/>
-      <c r="W91" s="173" t="n"/>
-      <c r="X91" s="173" t="n"/>
-      <c r="Y91" s="173" t="n"/>
-    </row>
-    <row r="92" ht="12.75" customHeight="1" s="122">
-      <c r="A92" s="173" t="n"/>
-      <c r="B92" s="173" t="n"/>
-      <c r="C92" s="173" t="n"/>
-      <c r="D92" s="173" t="n"/>
-      <c r="E92" s="173" t="n"/>
-      <c r="F92" s="173" t="n"/>
-      <c r="G92" s="173" t="n"/>
-      <c r="H92" s="173" t="n"/>
-      <c r="I92" s="173" t="n"/>
-      <c r="J92" s="173" t="n"/>
-      <c r="K92" s="173" t="n"/>
-      <c r="L92" s="173" t="n"/>
-      <c r="M92" s="173" t="n"/>
-      <c r="N92" s="173" t="n"/>
-      <c r="O92" s="173" t="n"/>
-      <c r="P92" s="173" t="n"/>
-      <c r="Q92" s="173" t="n"/>
-      <c r="R92" s="173" t="n"/>
-      <c r="S92" s="173" t="n"/>
-      <c r="T92" s="173" t="n"/>
-      <c r="U92" s="173" t="n"/>
-      <c r="V92" s="173" t="n"/>
-      <c r="W92" s="173" t="n"/>
-      <c r="X92" s="173" t="n"/>
-      <c r="Y92" s="173" t="n"/>
-    </row>
-    <row r="93" ht="12.75" customHeight="1" s="122">
-      <c r="A93" s="173" t="n"/>
-      <c r="B93" s="173" t="n"/>
-      <c r="C93" s="173" t="n"/>
-      <c r="D93" s="173" t="n"/>
-      <c r="E93" s="173" t="n"/>
-      <c r="F93" s="173" t="n"/>
-      <c r="G93" s="173" t="n"/>
-      <c r="H93" s="173" t="n"/>
-      <c r="I93" s="173" t="n"/>
-      <c r="J93" s="173" t="n"/>
-      <c r="K93" s="173" t="n"/>
-      <c r="L93" s="173" t="n"/>
-      <c r="M93" s="173" t="n"/>
-      <c r="N93" s="173" t="n"/>
-      <c r="O93" s="173" t="n"/>
-      <c r="P93" s="173" t="n"/>
-      <c r="Q93" s="173" t="n"/>
-      <c r="R93" s="173" t="n"/>
-      <c r="S93" s="173" t="n"/>
-      <c r="T93" s="173" t="n"/>
-      <c r="U93" s="173" t="n"/>
-      <c r="V93" s="173" t="n"/>
-      <c r="W93" s="173" t="n"/>
-      <c r="X93" s="173" t="n"/>
-      <c r="Y93" s="173" t="n"/>
-    </row>
-    <row r="94" ht="12.75" customHeight="1" s="122">
-      <c r="A94" s="173" t="n"/>
-      <c r="B94" s="173" t="n"/>
-      <c r="C94" s="173" t="n"/>
-      <c r="D94" s="173" t="n"/>
-      <c r="E94" s="173" t="n"/>
-      <c r="F94" s="173" t="n"/>
-      <c r="G94" s="173" t="n"/>
-      <c r="H94" s="173" t="n"/>
-      <c r="I94" s="173" t="n"/>
-      <c r="J94" s="173" t="n"/>
-      <c r="K94" s="173" t="n"/>
-      <c r="L94" s="173" t="n"/>
-      <c r="M94" s="173" t="n"/>
-      <c r="N94" s="173" t="n"/>
-      <c r="O94" s="173" t="n"/>
-      <c r="P94" s="173" t="n"/>
-      <c r="Q94" s="173" t="n"/>
-      <c r="R94" s="173" t="n"/>
-      <c r="S94" s="173" t="n"/>
-      <c r="T94" s="173" t="n"/>
-      <c r="U94" s="173" t="n"/>
-      <c r="V94" s="173" t="n"/>
-      <c r="W94" s="173" t="n"/>
-      <c r="X94" s="173" t="n"/>
-      <c r="Y94" s="173" t="n"/>
-    </row>
-    <row r="95" ht="12.75" customHeight="1" s="122">
-      <c r="A95" s="173" t="n"/>
-      <c r="B95" s="173" t="n"/>
-      <c r="C95" s="173" t="n"/>
-      <c r="D95" s="173" t="n"/>
-      <c r="E95" s="173" t="n"/>
-      <c r="F95" s="173" t="n"/>
-      <c r="G95" s="173" t="n"/>
-      <c r="H95" s="173" t="n"/>
-      <c r="I95" s="173" t="n"/>
-      <c r="J95" s="173" t="n"/>
-      <c r="K95" s="173" t="n"/>
-      <c r="L95" s="173" t="n"/>
-      <c r="M95" s="173" t="n"/>
-      <c r="N95" s="173" t="n"/>
-      <c r="O95" s="173" t="n"/>
-      <c r="P95" s="173" t="n"/>
-      <c r="Q95" s="173" t="n"/>
-      <c r="R95" s="173" t="n"/>
-      <c r="S95" s="173" t="n"/>
-      <c r="T95" s="173" t="n"/>
-      <c r="U95" s="173" t="n"/>
-      <c r="V95" s="173" t="n"/>
-      <c r="W95" s="173" t="n"/>
-      <c r="X95" s="173" t="n"/>
-      <c r="Y95" s="173" t="n"/>
-    </row>
-    <row r="96" ht="12.75" customHeight="1" s="122">
-      <c r="A96" s="173" t="n"/>
-      <c r="B96" s="173" t="n"/>
-      <c r="C96" s="173" t="n"/>
-      <c r="D96" s="173" t="n"/>
-      <c r="E96" s="173" t="n"/>
-      <c r="F96" s="173" t="n"/>
-      <c r="G96" s="173" t="n"/>
-      <c r="H96" s="173" t="n"/>
-      <c r="I96" s="173" t="n"/>
-      <c r="J96" s="173" t="n"/>
-      <c r="K96" s="173" t="n"/>
-      <c r="L96" s="173" t="n"/>
-      <c r="M96" s="173" t="n"/>
-      <c r="N96" s="173" t="n"/>
-      <c r="O96" s="173" t="n"/>
-      <c r="P96" s="173" t="n"/>
-      <c r="Q96" s="173" t="n"/>
-      <c r="R96" s="173" t="n"/>
-      <c r="S96" s="173" t="n"/>
-      <c r="T96" s="173" t="n"/>
-      <c r="U96" s="173" t="n"/>
-      <c r="V96" s="173" t="n"/>
-      <c r="W96" s="173" t="n"/>
-      <c r="X96" s="173" t="n"/>
-      <c r="Y96" s="173" t="n"/>
-    </row>
-    <row r="97" ht="12.75" customHeight="1" s="122">
-      <c r="A97" s="173" t="n"/>
-      <c r="B97" s="173" t="n"/>
-      <c r="C97" s="173" t="n"/>
-      <c r="D97" s="173" t="n"/>
-      <c r="E97" s="173" t="n"/>
-      <c r="F97" s="173" t="n"/>
-      <c r="G97" s="173" t="n"/>
-      <c r="H97" s="173" t="n"/>
-      <c r="I97" s="173" t="n"/>
-      <c r="J97" s="173" t="n"/>
-      <c r="K97" s="173" t="n"/>
-      <c r="L97" s="173" t="n"/>
-      <c r="M97" s="173" t="n"/>
-      <c r="N97" s="173" t="n"/>
-      <c r="O97" s="173" t="n"/>
-      <c r="P97" s="173" t="n"/>
-      <c r="Q97" s="173" t="n"/>
-      <c r="R97" s="173" t="n"/>
-      <c r="S97" s="173" t="n"/>
-      <c r="T97" s="173" t="n"/>
-      <c r="U97" s="173" t="n"/>
-      <c r="V97" s="173" t="n"/>
-      <c r="W97" s="173" t="n"/>
-      <c r="X97" s="173" t="n"/>
-      <c r="Y97" s="173" t="n"/>
-    </row>
-    <row r="98" ht="12.75" customHeight="1" s="122">
-      <c r="A98" s="173" t="n"/>
-      <c r="B98" s="173" t="n"/>
-      <c r="C98" s="173" t="n"/>
-      <c r="D98" s="173" t="n"/>
-      <c r="E98" s="173" t="n"/>
-      <c r="F98" s="173" t="n"/>
-      <c r="G98" s="173" t="n"/>
-      <c r="H98" s="173" t="n"/>
-      <c r="I98" s="173" t="n"/>
-      <c r="J98" s="173" t="n"/>
-      <c r="K98" s="173" t="n"/>
-      <c r="L98" s="173" t="n"/>
-      <c r="M98" s="173" t="n"/>
-      <c r="N98" s="173" t="n"/>
-      <c r="O98" s="173" t="n"/>
-      <c r="P98" s="173" t="n"/>
-      <c r="Q98" s="173" t="n"/>
-      <c r="R98" s="173" t="n"/>
-      <c r="S98" s="173" t="n"/>
-      <c r="T98" s="173" t="n"/>
-      <c r="U98" s="173" t="n"/>
-      <c r="V98" s="173" t="n"/>
-      <c r="W98" s="173" t="n"/>
-      <c r="X98" s="173" t="n"/>
-      <c r="Y98" s="173" t="n"/>
-    </row>
-    <row r="99" ht="12.75" customHeight="1" s="122">
-      <c r="A99" s="173" t="n"/>
-      <c r="B99" s="173" t="n"/>
-      <c r="C99" s="173" t="n"/>
-      <c r="D99" s="173" t="n"/>
-      <c r="E99" s="173" t="n"/>
-      <c r="F99" s="173" t="n"/>
-      <c r="G99" s="173" t="n"/>
-      <c r="H99" s="173" t="n"/>
-      <c r="I99" s="173" t="n"/>
-      <c r="J99" s="173" t="n"/>
-      <c r="K99" s="173" t="n"/>
-      <c r="L99" s="173" t="n"/>
-      <c r="M99" s="173" t="n"/>
-      <c r="N99" s="173" t="n"/>
-      <c r="O99" s="173" t="n"/>
-      <c r="P99" s="173" t="n"/>
-      <c r="Q99" s="173" t="n"/>
-      <c r="R99" s="173" t="n"/>
-      <c r="S99" s="173" t="n"/>
-      <c r="T99" s="173" t="n"/>
-      <c r="U99" s="173" t="n"/>
-      <c r="V99" s="173" t="n"/>
-      <c r="W99" s="173" t="n"/>
-      <c r="X99" s="173" t="n"/>
-      <c r="Y99" s="173" t="n"/>
-    </row>
-    <row r="100" ht="12.75" customHeight="1" s="122">
-      <c r="A100" s="173" t="n"/>
-      <c r="B100" s="173" t="n"/>
-      <c r="C100" s="173" t="n"/>
-      <c r="D100" s="173" t="n"/>
-      <c r="E100" s="173" t="n"/>
-      <c r="F100" s="173" t="n"/>
-      <c r="G100" s="173" t="n"/>
-      <c r="H100" s="173" t="n"/>
-      <c r="I100" s="173" t="n"/>
-      <c r="J100" s="173" t="n"/>
-      <c r="K100" s="173" t="n"/>
-      <c r="L100" s="173" t="n"/>
-      <c r="M100" s="173" t="n"/>
-      <c r="N100" s="173" t="n"/>
-      <c r="O100" s="173" t="n"/>
-      <c r="P100" s="173" t="n"/>
-      <c r="Q100" s="173" t="n"/>
-      <c r="R100" s="173" t="n"/>
-      <c r="S100" s="173" t="n"/>
-      <c r="T100" s="173" t="n"/>
-      <c r="U100" s="173" t="n"/>
-      <c r="V100" s="173" t="n"/>
-      <c r="W100" s="173" t="n"/>
-      <c r="X100" s="173" t="n"/>
-      <c r="Y100" s="173" t="n"/>
-    </row>
-    <row r="101" ht="12.75" customHeight="1" s="122">
-      <c r="A101" s="173" t="n"/>
-      <c r="B101" s="173" t="n"/>
-      <c r="C101" s="173" t="n"/>
-      <c r="D101" s="173" t="n"/>
-      <c r="E101" s="173" t="n"/>
-      <c r="F101" s="173" t="n"/>
-      <c r="G101" s="173" t="n"/>
-      <c r="H101" s="173" t="n"/>
-      <c r="I101" s="173" t="n"/>
-      <c r="J101" s="173" t="n"/>
-      <c r="K101" s="173" t="n"/>
-      <c r="L101" s="173" t="n"/>
-      <c r="M101" s="173" t="n"/>
-      <c r="N101" s="173" t="n"/>
-      <c r="O101" s="173" t="n"/>
-      <c r="P101" s="173" t="n"/>
-      <c r="Q101" s="173" t="n"/>
-      <c r="R101" s="173" t="n"/>
-      <c r="S101" s="173" t="n"/>
-      <c r="T101" s="173" t="n"/>
-      <c r="U101" s="173" t="n"/>
-      <c r="V101" s="173" t="n"/>
-      <c r="W101" s="173" t="n"/>
-      <c r="X101" s="173" t="n"/>
-      <c r="Y101" s="173" t="n"/>
-    </row>
-    <row r="102" ht="12.75" customHeight="1" s="122">
-      <c r="A102" s="173" t="n"/>
-      <c r="B102" s="173" t="n"/>
-      <c r="C102" s="173" t="n"/>
-      <c r="D102" s="173" t="n"/>
-      <c r="E102" s="173" t="n"/>
-      <c r="F102" s="173" t="n"/>
-      <c r="G102" s="173" t="n"/>
-      <c r="H102" s="173" t="n"/>
-      <c r="I102" s="173" t="n"/>
-      <c r="J102" s="173" t="n"/>
-      <c r="K102" s="173" t="n"/>
-      <c r="L102" s="173" t="n"/>
-      <c r="M102" s="173" t="n"/>
-      <c r="N102" s="173" t="n"/>
-      <c r="O102" s="173" t="n"/>
-      <c r="P102" s="173" t="n"/>
-      <c r="Q102" s="173" t="n"/>
-      <c r="R102" s="173" t="n"/>
-      <c r="S102" s="173" t="n"/>
-      <c r="T102" s="173" t="n"/>
-      <c r="U102" s="173" t="n"/>
-      <c r="V102" s="173" t="n"/>
-      <c r="W102" s="173" t="n"/>
-      <c r="X102" s="173" t="n"/>
-      <c r="Y102" s="173" t="n"/>
-    </row>
-    <row r="103" ht="12.75" customHeight="1" s="122">
-      <c r="A103" s="173" t="n"/>
-      <c r="B103" s="173" t="n"/>
-      <c r="C103" s="173" t="n"/>
-      <c r="D103" s="173" t="n"/>
-      <c r="E103" s="173" t="n"/>
-      <c r="F103" s="173" t="n"/>
-      <c r="G103" s="173" t="n"/>
-      <c r="H103" s="173" t="n"/>
-      <c r="I103" s="173" t="n"/>
-      <c r="J103" s="173" t="n"/>
-      <c r="K103" s="173" t="n"/>
-      <c r="L103" s="173" t="n"/>
-      <c r="M103" s="173" t="n"/>
-      <c r="N103" s="173" t="n"/>
-      <c r="O103" s="173" t="n"/>
-      <c r="P103" s="173" t="n"/>
-      <c r="Q103" s="173" t="n"/>
-      <c r="R103" s="173" t="n"/>
-      <c r="S103" s="173" t="n"/>
-      <c r="T103" s="173" t="n"/>
-      <c r="U103" s="173" t="n"/>
-      <c r="V103" s="173" t="n"/>
-      <c r="W103" s="173" t="n"/>
-      <c r="X103" s="173" t="n"/>
-      <c r="Y103" s="173" t="n"/>
-    </row>
-    <row r="104" ht="12.75" customHeight="1" s="122">
-      <c r="A104" s="173" t="n"/>
-      <c r="B104" s="173" t="n"/>
-      <c r="C104" s="173" t="n"/>
-      <c r="D104" s="173" t="n"/>
-      <c r="E104" s="173" t="n"/>
-      <c r="F104" s="173" t="n"/>
-      <c r="G104" s="173" t="n"/>
-      <c r="H104" s="173" t="n"/>
-      <c r="I104" s="173" t="n"/>
-      <c r="J104" s="173" t="n"/>
-      <c r="K104" s="173" t="n"/>
-      <c r="L104" s="173" t="n"/>
-      <c r="M104" s="173" t="n"/>
-      <c r="N104" s="173" t="n"/>
-      <c r="O104" s="173" t="n"/>
-      <c r="P104" s="173" t="n"/>
-      <c r="Q104" s="173" t="n"/>
-      <c r="R104" s="173" t="n"/>
-      <c r="S104" s="173" t="n"/>
-      <c r="T104" s="173" t="n"/>
-      <c r="U104" s="173" t="n"/>
-      <c r="V104" s="173" t="n"/>
-      <c r="W104" s="173" t="n"/>
-      <c r="X104" s="173" t="n"/>
-      <c r="Y104" s="173" t="n"/>
-    </row>
-    <row r="105" ht="12.75" customHeight="1" s="122">
-      <c r="A105" s="173" t="n"/>
-      <c r="B105" s="173" t="n"/>
-      <c r="C105" s="173" t="n"/>
-      <c r="D105" s="173" t="n"/>
-      <c r="E105" s="173" t="n"/>
-      <c r="F105" s="173" t="n"/>
-      <c r="G105" s="173" t="n"/>
-      <c r="H105" s="173" t="n"/>
-      <c r="I105" s="173" t="n"/>
-      <c r="J105" s="173" t="n"/>
-      <c r="K105" s="173" t="n"/>
-      <c r="L105" s="173" t="n"/>
-      <c r="M105" s="173" t="n"/>
-      <c r="N105" s="173" t="n"/>
-      <c r="O105" s="173" t="n"/>
-      <c r="P105" s="173" t="n"/>
-      <c r="Q105" s="173" t="n"/>
-      <c r="R105" s="173" t="n"/>
-      <c r="S105" s="173" t="n"/>
-      <c r="T105" s="173" t="n"/>
-      <c r="U105" s="173" t="n"/>
-      <c r="V105" s="173" t="n"/>
-      <c r="W105" s="173" t="n"/>
-      <c r="X105" s="173" t="n"/>
-      <c r="Y105" s="173" t="n"/>
-    </row>
-    <row r="106" ht="12.75" customHeight="1" s="122">
-      <c r="A106" s="173" t="n"/>
-      <c r="B106" s="173" t="n"/>
-      <c r="C106" s="173" t="n"/>
-      <c r="D106" s="173" t="n"/>
-      <c r="E106" s="173" t="n"/>
-      <c r="F106" s="173" t="n"/>
-      <c r="G106" s="173" t="n"/>
-      <c r="H106" s="173" t="n"/>
-      <c r="I106" s="173" t="n"/>
-      <c r="J106" s="173" t="n"/>
-      <c r="K106" s="173" t="n"/>
-      <c r="L106" s="173" t="n"/>
-      <c r="M106" s="173" t="n"/>
-      <c r="N106" s="173" t="n"/>
-      <c r="O106" s="173" t="n"/>
-      <c r="P106" s="173" t="n"/>
-      <c r="Q106" s="173" t="n"/>
-      <c r="R106" s="173" t="n"/>
-      <c r="S106" s="173" t="n"/>
-      <c r="T106" s="173" t="n"/>
-      <c r="U106" s="173" t="n"/>
-      <c r="V106" s="173" t="n"/>
-      <c r="W106" s="173" t="n"/>
-      <c r="X106" s="173" t="n"/>
-      <c r="Y106" s="173" t="n"/>
-    </row>
-    <row r="107" ht="17.25" customHeight="1" s="122">
-      <c r="A107" s="173" t="n"/>
-      <c r="B107" s="173" t="n"/>
-      <c r="C107" s="173" t="n"/>
-      <c r="D107" s="173" t="n"/>
-      <c r="E107" s="173" t="n"/>
-      <c r="F107" s="173" t="n"/>
-      <c r="G107" s="173" t="n"/>
-      <c r="H107" s="173" t="n"/>
-      <c r="I107" s="173" t="n"/>
-      <c r="J107" s="173" t="n"/>
-      <c r="K107" s="173" t="n"/>
-      <c r="L107" s="173" t="n"/>
-      <c r="M107" s="173" t="n"/>
-      <c r="N107" s="173" t="n"/>
-      <c r="O107" s="173" t="n"/>
-      <c r="P107" s="173" t="n"/>
-      <c r="Q107" s="173" t="n"/>
-      <c r="R107" s="173" t="n"/>
-      <c r="S107" s="173" t="n"/>
-      <c r="T107" s="173" t="n"/>
-      <c r="U107" s="173" t="n"/>
-      <c r="V107" s="173" t="n"/>
-      <c r="W107" s="173" t="n"/>
-      <c r="X107" s="173" t="n"/>
-      <c r="Y107" s="173" t="n"/>
-    </row>
-    <row r="108" ht="17.25" customHeight="1" s="122">
-      <c r="A108" s="173" t="n"/>
-      <c r="B108" s="173" t="n"/>
-      <c r="C108" s="173" t="n"/>
-      <c r="D108" s="173" t="n"/>
-      <c r="E108" s="173" t="n"/>
-      <c r="F108" s="173" t="n"/>
-      <c r="G108" s="173" t="n"/>
-      <c r="H108" s="173" t="n"/>
-      <c r="I108" s="173" t="n"/>
-      <c r="J108" s="173" t="n"/>
-      <c r="K108" s="173" t="n"/>
-      <c r="L108" s="173" t="n"/>
-      <c r="M108" s="173" t="n"/>
-      <c r="N108" s="173" t="n"/>
-      <c r="O108" s="173" t="n"/>
-      <c r="P108" s="173" t="n"/>
-      <c r="Q108" s="173" t="n"/>
-      <c r="R108" s="173" t="n"/>
-      <c r="S108" s="173" t="n"/>
-      <c r="T108" s="173" t="n"/>
-      <c r="U108" s="173" t="n"/>
-      <c r="V108" s="173" t="n"/>
-      <c r="W108" s="173" t="n"/>
-      <c r="X108" s="173" t="n"/>
-      <c r="Y108" s="173" t="n"/>
-    </row>
-    <row r="109" ht="17.25" customHeight="1" s="122">
-      <c r="A109" s="173" t="n"/>
-      <c r="B109" s="173" t="n"/>
-      <c r="C109" s="173" t="n"/>
-      <c r="D109" s="173" t="n"/>
-      <c r="E109" s="173" t="n"/>
-      <c r="F109" s="173" t="n"/>
-      <c r="G109" s="173" t="n"/>
-      <c r="H109" s="173" t="n"/>
-      <c r="I109" s="173" t="n"/>
-      <c r="J109" s="173" t="n"/>
-      <c r="K109" s="173" t="n"/>
-      <c r="L109" s="173" t="n"/>
-      <c r="M109" s="173" t="n"/>
-      <c r="N109" s="173" t="n"/>
-      <c r="O109" s="173" t="n"/>
-      <c r="P109" s="173" t="n"/>
-      <c r="Q109" s="173" t="n"/>
-      <c r="R109" s="173" t="n"/>
-      <c r="S109" s="173" t="n"/>
-      <c r="T109" s="173" t="n"/>
-      <c r="U109" s="173" t="n"/>
-      <c r="V109" s="173" t="n"/>
-      <c r="W109" s="173" t="n"/>
-      <c r="X109" s="173" t="n"/>
-      <c r="Y109" s="173" t="n"/>
-    </row>
-    <row r="110" ht="17.25" customHeight="1" s="122">
-      <c r="A110" s="173" t="n"/>
-      <c r="B110" s="173" t="n"/>
-      <c r="C110" s="173" t="n"/>
-      <c r="D110" s="173" t="n"/>
-      <c r="E110" s="173" t="n"/>
-      <c r="F110" s="173" t="n"/>
-      <c r="G110" s="173" t="n"/>
-      <c r="H110" s="173" t="n"/>
-      <c r="I110" s="173" t="n"/>
-      <c r="J110" s="173" t="n"/>
-      <c r="K110" s="173" t="n"/>
-      <c r="L110" s="173" t="n"/>
-      <c r="M110" s="173" t="n"/>
-      <c r="N110" s="173" t="n"/>
-      <c r="O110" s="173" t="n"/>
-      <c r="P110" s="173" t="n"/>
-      <c r="Q110" s="173" t="n"/>
-      <c r="R110" s="173" t="n"/>
-      <c r="S110" s="173" t="n"/>
-      <c r="T110" s="173" t="n"/>
-      <c r="U110" s="173" t="n"/>
-      <c r="V110" s="173" t="n"/>
-      <c r="W110" s="173" t="n"/>
-      <c r="X110" s="173" t="n"/>
-      <c r="Y110" s="173" t="n"/>
-    </row>
-    <row r="111" ht="17.25" customHeight="1" s="122">
-      <c r="A111" s="173" t="n"/>
-      <c r="B111" s="173" t="n"/>
-      <c r="C111" s="173" t="n"/>
-      <c r="D111" s="173" t="n"/>
-      <c r="E111" s="173" t="n"/>
-      <c r="F111" s="173" t="n"/>
-      <c r="G111" s="173" t="n"/>
-      <c r="H111" s="173" t="n"/>
-      <c r="I111" s="173" t="n"/>
-      <c r="J111" s="173" t="n"/>
-      <c r="K111" s="173" t="n"/>
-      <c r="L111" s="173" t="n"/>
-      <c r="M111" s="173" t="n"/>
-      <c r="N111" s="173" t="n"/>
-      <c r="O111" s="173" t="n"/>
-      <c r="P111" s="173" t="n"/>
-      <c r="Q111" s="173" t="n"/>
-      <c r="R111" s="173" t="n"/>
-      <c r="S111" s="173" t="n"/>
-      <c r="T111" s="173" t="n"/>
-      <c r="U111" s="173" t="n"/>
-      <c r="V111" s="173" t="n"/>
-      <c r="W111" s="173" t="n"/>
-      <c r="X111" s="173" t="n"/>
-      <c r="Y111" s="173" t="n"/>
-    </row>
-    <row r="112" ht="17.25" customHeight="1" s="122">
-      <c r="A112" s="173" t="n"/>
-      <c r="B112" s="173" t="n"/>
-      <c r="C112" s="173" t="n"/>
-      <c r="D112" s="173" t="n"/>
-      <c r="E112" s="173" t="n"/>
-      <c r="F112" s="173" t="n"/>
-      <c r="G112" s="173" t="n"/>
-      <c r="H112" s="173" t="n"/>
-      <c r="I112" s="173" t="n"/>
-      <c r="J112" s="173" t="n"/>
-      <c r="K112" s="173" t="n"/>
-      <c r="L112" s="173" t="n"/>
-      <c r="M112" s="173" t="n"/>
-      <c r="N112" s="173" t="n"/>
-      <c r="O112" s="173" t="n"/>
-      <c r="P112" s="173" t="n"/>
-      <c r="Q112" s="173" t="n"/>
-      <c r="R112" s="173" t="n"/>
-      <c r="S112" s="173" t="n"/>
-      <c r="T112" s="173" t="n"/>
-      <c r="U112" s="173" t="n"/>
-      <c r="V112" s="173" t="n"/>
-      <c r="W112" s="173" t="n"/>
-      <c r="X112" s="173" t="n"/>
-      <c r="Y112" s="173" t="n"/>
-    </row>
-    <row r="113" ht="17.25" customHeight="1" s="122">
-      <c r="A113" s="173" t="n"/>
-      <c r="B113" s="173" t="n"/>
-      <c r="C113" s="173" t="n"/>
-      <c r="D113" s="173" t="n"/>
-      <c r="E113" s="173" t="n"/>
-      <c r="F113" s="173" t="n"/>
-      <c r="G113" s="173" t="n"/>
-      <c r="H113" s="173" t="n"/>
-      <c r="I113" s="173" t="n"/>
-      <c r="J113" s="173" t="n"/>
-      <c r="K113" s="173" t="n"/>
-      <c r="L113" s="173" t="n"/>
-      <c r="M113" s="173" t="n"/>
-      <c r="N113" s="173" t="n"/>
-      <c r="O113" s="173" t="n"/>
-      <c r="P113" s="173" t="n"/>
-      <c r="Q113" s="173" t="n"/>
-      <c r="R113" s="173" t="n"/>
-      <c r="S113" s="173" t="n"/>
-      <c r="T113" s="173" t="n"/>
-      <c r="U113" s="173" t="n"/>
-      <c r="V113" s="173" t="n"/>
-      <c r="W113" s="173" t="n"/>
-      <c r="X113" s="173" t="n"/>
-      <c r="Y113" s="173" t="n"/>
-    </row>
-    <row r="114" ht="17.25" customHeight="1" s="122">
-      <c r="A114" s="173" t="n"/>
-      <c r="B114" s="173" t="n"/>
-      <c r="C114" s="173" t="n"/>
-      <c r="D114" s="173" t="n"/>
-      <c r="E114" s="173" t="n"/>
-      <c r="F114" s="173" t="n"/>
-      <c r="G114" s="173" t="n"/>
-      <c r="H114" s="173" t="n"/>
-      <c r="I114" s="173" t="n"/>
-      <c r="J114" s="173" t="n"/>
-      <c r="K114" s="173" t="n"/>
-      <c r="L114" s="173" t="n"/>
-      <c r="M114" s="173" t="n"/>
-      <c r="N114" s="173" t="n"/>
-      <c r="O114" s="173" t="n"/>
-      <c r="P114" s="173" t="n"/>
-      <c r="Q114" s="173" t="n"/>
-      <c r="R114" s="173" t="n"/>
-      <c r="S114" s="173" t="n"/>
-      <c r="T114" s="173" t="n"/>
-      <c r="U114" s="173" t="n"/>
-      <c r="V114" s="173" t="n"/>
-      <c r="W114" s="173" t="n"/>
-      <c r="X114" s="173" t="n"/>
-      <c r="Y114" s="173" t="n"/>
-    </row>
-    <row r="115" ht="17.25" customHeight="1" s="122">
-      <c r="A115" s="173" t="n"/>
-      <c r="B115" s="173" t="n"/>
-      <c r="C115" s="173" t="n"/>
-      <c r="D115" s="173" t="n"/>
-      <c r="E115" s="173" t="n"/>
-      <c r="F115" s="173" t="n"/>
-      <c r="G115" s="173" t="n"/>
-      <c r="H115" s="173" t="n"/>
-      <c r="I115" s="173" t="n"/>
-      <c r="J115" s="173" t="n"/>
-      <c r="K115" s="173" t="n"/>
-      <c r="L115" s="173" t="n"/>
-      <c r="M115" s="173" t="n"/>
-      <c r="N115" s="173" t="n"/>
-      <c r="O115" s="173" t="n"/>
-      <c r="P115" s="173" t="n"/>
-      <c r="Q115" s="173" t="n"/>
-      <c r="R115" s="173" t="n"/>
-      <c r="S115" s="173" t="n"/>
-      <c r="T115" s="173" t="n"/>
-      <c r="U115" s="173" t="n"/>
-      <c r="V115" s="173" t="n"/>
-      <c r="W115" s="173" t="n"/>
-      <c r="X115" s="173" t="n"/>
-      <c r="Y115" s="173" t="n"/>
-    </row>
-    <row r="116" ht="17.25" customHeight="1" s="122">
-      <c r="A116" s="173" t="n"/>
-      <c r="B116" s="173" t="n"/>
-      <c r="C116" s="173" t="n"/>
-      <c r="D116" s="173" t="n"/>
-      <c r="E116" s="173" t="n"/>
-      <c r="F116" s="173" t="n"/>
-      <c r="G116" s="173" t="n"/>
-      <c r="H116" s="173" t="n"/>
-      <c r="I116" s="173" t="n"/>
-      <c r="J116" s="173" t="n"/>
-      <c r="K116" s="173" t="n"/>
-      <c r="L116" s="173" t="n"/>
-      <c r="M116" s="173" t="n"/>
-      <c r="N116" s="173" t="n"/>
-      <c r="O116" s="173" t="n"/>
-      <c r="P116" s="173" t="n"/>
-      <c r="Q116" s="173" t="n"/>
-      <c r="R116" s="173" t="n"/>
-      <c r="S116" s="173" t="n"/>
-      <c r="T116" s="173" t="n"/>
-      <c r="U116" s="173" t="n"/>
-      <c r="V116" s="173" t="n"/>
-      <c r="W116" s="173" t="n"/>
-      <c r="X116" s="173" t="n"/>
-      <c r="Y116" s="173" t="n"/>
-    </row>
-    <row r="117" ht="17.25" customHeight="1" s="122">
-      <c r="A117" s="173" t="n"/>
-      <c r="B117" s="173" t="n"/>
-      <c r="C117" s="173" t="n"/>
-      <c r="D117" s="173" t="n"/>
-      <c r="E117" s="173" t="n"/>
-      <c r="F117" s="173" t="n"/>
-      <c r="G117" s="173" t="n"/>
-      <c r="H117" s="173" t="n"/>
-      <c r="I117" s="173" t="n"/>
-      <c r="J117" s="173" t="n"/>
-      <c r="K117" s="173" t="n"/>
-      <c r="L117" s="173" t="n"/>
-      <c r="M117" s="173" t="n"/>
-      <c r="N117" s="173" t="n"/>
-      <c r="O117" s="173" t="n"/>
-      <c r="P117" s="173" t="n"/>
-      <c r="Q117" s="173" t="n"/>
-      <c r="R117" s="173" t="n"/>
-      <c r="S117" s="173" t="n"/>
-      <c r="T117" s="173" t="n"/>
-      <c r="U117" s="173" t="n"/>
-      <c r="V117" s="173" t="n"/>
-      <c r="W117" s="173" t="n"/>
-      <c r="X117" s="173" t="n"/>
-      <c r="Y117" s="173" t="n"/>
-    </row>
-    <row r="118" ht="17.25" customHeight="1" s="122">
-      <c r="A118" s="173" t="n"/>
-      <c r="B118" s="173" t="n"/>
-      <c r="C118" s="173" t="n"/>
-      <c r="D118" s="173" t="n"/>
-      <c r="E118" s="173" t="n"/>
-      <c r="F118" s="173" t="n"/>
-      <c r="G118" s="173" t="n"/>
-      <c r="H118" s="173" t="n"/>
-      <c r="I118" s="173" t="n"/>
-      <c r="J118" s="173" t="n"/>
-      <c r="K118" s="173" t="n"/>
-      <c r="L118" s="173" t="n"/>
-      <c r="M118" s="173" t="n"/>
-      <c r="N118" s="173" t="n"/>
-      <c r="O118" s="173" t="n"/>
-      <c r="P118" s="173" t="n"/>
-      <c r="Q118" s="173" t="n"/>
-      <c r="R118" s="173" t="n"/>
-      <c r="S118" s="173" t="n"/>
-      <c r="T118" s="173" t="n"/>
-      <c r="U118" s="173" t="n"/>
-      <c r="V118" s="173" t="n"/>
-      <c r="W118" s="173" t="n"/>
-      <c r="X118" s="173" t="n"/>
-      <c r="Y118" s="173" t="n"/>
-    </row>
-    <row r="119" ht="17.25" customHeight="1" s="122">
-      <c r="A119" s="173" t="n"/>
-      <c r="B119" s="173" t="n"/>
-      <c r="C119" s="173" t="n"/>
-      <c r="D119" s="173" t="n"/>
-      <c r="E119" s="173" t="n"/>
-      <c r="F119" s="173" t="n"/>
-      <c r="G119" s="173" t="n"/>
-      <c r="H119" s="173" t="n"/>
-      <c r="I119" s="173" t="n"/>
-      <c r="J119" s="173" t="n"/>
-      <c r="K119" s="173" t="n"/>
-      <c r="L119" s="173" t="n"/>
-      <c r="M119" s="173" t="n"/>
-      <c r="N119" s="173" t="n"/>
-      <c r="O119" s="173" t="n"/>
-      <c r="P119" s="173" t="n"/>
-      <c r="Q119" s="173" t="n"/>
-      <c r="R119" s="173" t="n"/>
-      <c r="S119" s="173" t="n"/>
-      <c r="T119" s="173" t="n"/>
-      <c r="U119" s="173" t="n"/>
-      <c r="V119" s="173" t="n"/>
-      <c r="W119" s="173" t="n"/>
-      <c r="X119" s="173" t="n"/>
-      <c r="Y119" s="173" t="n"/>
-    </row>
-    <row r="120" ht="17.25" customHeight="1" s="122">
-      <c r="A120" s="173" t="n"/>
-      <c r="B120" s="173" t="n"/>
-      <c r="C120" s="173" t="n"/>
-      <c r="D120" s="173" t="n"/>
-      <c r="E120" s="173" t="n"/>
-      <c r="F120" s="173" t="n"/>
-      <c r="G120" s="173" t="n"/>
-      <c r="H120" s="173" t="n"/>
-      <c r="I120" s="173" t="n"/>
-      <c r="J120" s="173" t="n"/>
-      <c r="K120" s="173" t="n"/>
-      <c r="L120" s="173" t="n"/>
-      <c r="M120" s="173" t="n"/>
-      <c r="N120" s="173" t="n"/>
-      <c r="O120" s="173" t="n"/>
-      <c r="P120" s="173" t="n"/>
-      <c r="Q120" s="173" t="n"/>
-      <c r="R120" s="173" t="n"/>
-      <c r="S120" s="173" t="n"/>
-      <c r="T120" s="173" t="n"/>
-      <c r="U120" s="173" t="n"/>
-      <c r="V120" s="173" t="n"/>
-      <c r="W120" s="173" t="n"/>
-      <c r="X120" s="173" t="n"/>
-      <c r="Y120" s="173" t="n"/>
-    </row>
-    <row r="121" ht="17.25" customHeight="1" s="122">
-      <c r="A121" s="173" t="n"/>
-      <c r="B121" s="173" t="n"/>
-      <c r="C121" s="173" t="n"/>
-      <c r="D121" s="173" t="n"/>
-      <c r="E121" s="173" t="n"/>
-      <c r="F121" s="173" t="n"/>
-      <c r="G121" s="173" t="n"/>
-      <c r="H121" s="173" t="n"/>
-      <c r="I121" s="173" t="n"/>
-      <c r="J121" s="173" t="n"/>
-      <c r="K121" s="173" t="n"/>
-      <c r="L121" s="173" t="n"/>
-      <c r="M121" s="173" t="n"/>
-      <c r="N121" s="173" t="n"/>
-      <c r="O121" s="173" t="n"/>
-      <c r="P121" s="173" t="n"/>
-      <c r="Q121" s="173" t="n"/>
-      <c r="R121" s="173" t="n"/>
-      <c r="S121" s="173" t="n"/>
-      <c r="T121" s="173" t="n"/>
-      <c r="U121" s="173" t="n"/>
-      <c r="V121" s="173" t="n"/>
-      <c r="W121" s="173" t="n"/>
-      <c r="X121" s="173" t="n"/>
-      <c r="Y121" s="173" t="n"/>
-    </row>
-    <row r="122" ht="9" customHeight="1" s="122"/>
-    <row r="123" ht="75" customHeight="1" s="122"/>
+    <row r="52" ht="9" customHeight="1" s="122"/>
+    <row r="53" ht="75" customHeight="1" s="122"/>
+    <row r="54" ht="12.75" customHeight="1" s="122"/>
+    <row r="55" ht="12.75" customHeight="1" s="122"/>
+    <row r="56" ht="12.75" customHeight="1" s="122"/>
+    <row r="57" ht="12.75" customHeight="1" s="122"/>
+    <row r="58" ht="12.75" customHeight="1" s="122"/>
+    <row r="59" ht="12.75" customHeight="1" s="122"/>
+    <row r="60" ht="12.75" customHeight="1" s="122"/>
+    <row r="61" ht="12.75" customHeight="1" s="122"/>
+    <row r="62" ht="12.75" customHeight="1" s="122"/>
+    <row r="63" ht="12.75" customHeight="1" s="122"/>
+    <row r="64" ht="12.75" customHeight="1" s="122"/>
+    <row r="65" ht="12.75" customHeight="1" s="122"/>
+    <row r="66" ht="12.75" customHeight="1" s="122"/>
+    <row r="67" ht="12.75" customHeight="1" s="122"/>
+    <row r="68" ht="12.75" customHeight="1" s="122"/>
+    <row r="69" ht="12.75" customHeight="1" s="122"/>
+    <row r="70" ht="12.75" customHeight="1" s="122"/>
+    <row r="71" ht="12.75" customHeight="1" s="122"/>
+    <row r="72" ht="12.75" customHeight="1" s="122"/>
+    <row r="73" ht="12.75" customHeight="1" s="122"/>
+    <row r="74" ht="12.75" customHeight="1" s="122"/>
+    <row r="75" ht="12.75" customHeight="1" s="122"/>
+    <row r="76" ht="12.75" customHeight="1" s="122"/>
+    <row r="77" ht="12.75" customHeight="1" s="122"/>
+    <row r="78" ht="12.75" customHeight="1" s="122"/>
+    <row r="79" ht="12.75" customHeight="1" s="122"/>
+    <row r="80" ht="12.75" customHeight="1" s="122"/>
+    <row r="81" ht="12.75" customHeight="1" s="122"/>
+    <row r="82" ht="12.75" customHeight="1" s="122"/>
+    <row r="83" ht="12.75" customHeight="1" s="122"/>
+    <row r="84" ht="12.75" customHeight="1" s="122"/>
+    <row r="85" ht="12.75" customHeight="1" s="122"/>
+    <row r="86" ht="12.75" customHeight="1" s="122"/>
+    <row r="87" ht="12.75" customHeight="1" s="122"/>
+    <row r="88" ht="12.75" customHeight="1" s="122"/>
+    <row r="89" ht="12.75" customHeight="1" s="122"/>
+    <row r="90" ht="12.75" customHeight="1" s="122"/>
+    <row r="91" ht="12.75" customHeight="1" s="122"/>
+    <row r="92" ht="12.75" customHeight="1" s="122"/>
+    <row r="93" ht="12.75" customHeight="1" s="122"/>
+    <row r="94" ht="12.75" customHeight="1" s="122"/>
+    <row r="95" ht="12.75" customHeight="1" s="122"/>
+    <row r="96" ht="12.75" customHeight="1" s="122"/>
+    <row r="97" ht="12.75" customHeight="1" s="122"/>
+    <row r="98" ht="12.75" customHeight="1" s="122"/>
+    <row r="99" ht="12.75" customHeight="1" s="122"/>
+    <row r="100" ht="12.75" customHeight="1" s="122"/>
+    <row r="101" ht="12.75" customHeight="1" s="122"/>
+    <row r="102" ht="12.75" customHeight="1" s="122"/>
+    <row r="103" ht="12.75" customHeight="1" s="122"/>
+    <row r="104" ht="12.75" customHeight="1" s="122"/>
+    <row r="105" ht="12.75" customHeight="1" s="122"/>
+    <row r="106" ht="12.75" customHeight="1" s="122"/>
+    <row r="107" ht="17.25" customHeight="1" s="122"/>
+    <row r="108" ht="17.25" customHeight="1" s="122"/>
+    <row r="109" ht="17.25" customHeight="1" s="122"/>
+    <row r="110" ht="17.25" customHeight="1" s="122"/>
+    <row r="111" ht="17.25" customHeight="1" s="122"/>
+    <row r="112" ht="17.25" customHeight="1" s="122"/>
+    <row r="113" ht="17.25" customHeight="1" s="122"/>
+    <row r="114" ht="17.25" customHeight="1" s="122"/>
+    <row r="115" ht="17.25" customHeight="1" s="122"/>
+    <row r="116" ht="17.25" customHeight="1" s="122"/>
+    <row r="117" ht="17.25" customHeight="1" s="122"/>
+    <row r="118" ht="17.25" customHeight="1" s="122"/>
+    <row r="119" ht="17.25" customHeight="1" s="122"/>
+    <row r="120" ht="17.25" customHeight="1" s="122"/>
+    <row r="121" ht="17.25" customHeight="1" s="122"/>
+    <row r="122" ht="17.25" customHeight="1" s="122"/>
+    <row r="123" ht="17.25" customHeight="1" s="122"/>
     <row r="124" ht="17.25" customHeight="1" s="122"/>
     <row r="125" ht="17.25" customHeight="1" s="122"/>
     <row r="126" ht="17.25" customHeight="1" s="122"/>
@@ -16719,7 +14716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN71"/>
+  <dimension ref="A1:AN52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="121" min="1" max="12"/>
@@ -18355,59 +16352,10 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="3" customHeight="1" s="122">
-      <c r="A51" s="204" t="n"/>
-      <c r="B51" s="204" t="n"/>
-      <c r="C51" s="204" t="n"/>
-      <c r="D51" s="204" t="n"/>
-      <c r="E51" s="204" t="n"/>
-      <c r="F51" s="204" t="n"/>
-      <c r="G51" s="204" t="n"/>
-      <c r="H51" s="204" t="n"/>
-      <c r="I51" s="204" t="n"/>
-      <c r="J51" s="204" t="n"/>
-      <c r="K51" s="204" t="n"/>
-      <c r="L51" s="204" t="n"/>
-      <c r="M51" s="204" t="n"/>
-      <c r="N51" s="204" t="n"/>
-      <c r="O51" s="204" t="n"/>
-      <c r="P51" s="204" t="n"/>
-      <c r="Q51" s="204" t="n"/>
-      <c r="R51" s="204" t="n"/>
-      <c r="S51" s="204" t="n"/>
-      <c r="T51" s="204" t="n"/>
-      <c r="U51" s="204" t="n"/>
-      <c r="V51" s="204" t="n"/>
-      <c r="W51" s="204" t="n"/>
-      <c r="X51" s="204" t="n"/>
-      <c r="Y51" s="204" t="n"/>
-      <c r="Z51" s="204" t="n"/>
-      <c r="AA51" s="121" t="n"/>
-      <c r="AB51" s="121" t="n"/>
-      <c r="AC51" s="121" t="n"/>
-      <c r="AD51" s="121" t="n"/>
-      <c r="AE51" s="121" t="n"/>
-      <c r="AF51" s="121" t="n"/>
-      <c r="AG51" s="121" t="n"/>
-      <c r="AH51" s="121" t="n"/>
-      <c r="AI51" s="121" t="n"/>
-      <c r="AJ51" s="121" t="n"/>
-    </row>
+    <row r="51" ht="9" customHeight="1" s="122"/>
+    <row r="52" ht="75" customHeight="1" s="122"/>
     <row r="68" ht="21" customHeight="1" s="122"/>
-    <row r="69" ht="13.5" customHeight="1" s="122">
-      <c r="A69" s="123" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN69" s="123" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="9" customHeight="1" s="122"/>
-    <row r="71" ht="75" customHeight="1" s="122"/>
+    <row r="69" ht="13.5" customHeight="1" s="122"/>
     <row r="110" ht="17.25" customHeight="1" s="122"/>
     <row r="111" ht="17.25" customHeight="1" s="122"/>
     <row r="112" ht="17.25" customHeight="1" s="122"/>
@@ -18673,7 +16621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN64"/>
+  <dimension ref="A1:AN61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="121" min="1" max="12"/>
@@ -21110,96 +19058,11 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="13.15" customFormat="1" customHeight="1" s="176">
-      <c r="A60" s="209" t="n"/>
-      <c r="B60" s="209" t="n"/>
-      <c r="C60" s="209" t="n"/>
-      <c r="D60" s="209" t="n"/>
-      <c r="E60" s="209" t="n"/>
-      <c r="F60" s="209" t="n"/>
-      <c r="G60" s="209" t="n"/>
-      <c r="H60" s="209" t="n"/>
-      <c r="I60" s="209" t="n"/>
-      <c r="J60" s="209" t="n"/>
-      <c r="K60" s="209" t="n"/>
-      <c r="L60" s="209" t="n"/>
-      <c r="M60" s="209" t="n"/>
-      <c r="N60" s="209" t="n"/>
-      <c r="O60" s="209" t="n"/>
-      <c r="P60" s="209" t="n"/>
-      <c r="Q60" s="209" t="n"/>
-      <c r="R60" s="209" t="n"/>
-      <c r="S60" s="209" t="n"/>
-      <c r="T60" s="209" t="n"/>
-      <c r="U60" s="209" t="n"/>
-      <c r="V60" s="209" t="n"/>
-      <c r="W60" s="209" t="n"/>
-      <c r="X60" s="209" t="n"/>
-      <c r="Y60" s="209" t="n"/>
-      <c r="Z60" s="209" t="n"/>
-      <c r="AA60" s="176" t="n"/>
-      <c r="AB60" s="176" t="n"/>
-      <c r="AC60" s="176" t="n"/>
-      <c r="AD60" s="176" t="n"/>
-      <c r="AE60" s="176" t="n"/>
-      <c r="AF60" s="176" t="n"/>
-      <c r="AG60" s="176" t="n"/>
-      <c r="AH60" s="176" t="n"/>
-      <c r="AI60" s="176" t="n"/>
-      <c r="AJ60" s="176" t="n"/>
-    </row>
-    <row r="61" ht="21" customFormat="1" customHeight="1" s="176">
-      <c r="A61" s="209" t="n"/>
-      <c r="B61" s="209" t="n"/>
-      <c r="C61" s="209" t="n"/>
-      <c r="D61" s="209" t="n"/>
-      <c r="E61" s="209" t="n"/>
-      <c r="F61" s="209" t="n"/>
-      <c r="G61" s="209" t="n"/>
-      <c r="H61" s="209" t="n"/>
-      <c r="I61" s="209" t="n"/>
-      <c r="J61" s="209" t="n"/>
-      <c r="K61" s="209" t="n"/>
-      <c r="L61" s="209" t="n"/>
-      <c r="M61" s="209" t="n"/>
-      <c r="N61" s="209" t="n"/>
-      <c r="O61" s="209" t="n"/>
-      <c r="P61" s="209" t="n"/>
-      <c r="Q61" s="209" t="n"/>
-      <c r="R61" s="209" t="n"/>
-      <c r="S61" s="209" t="n"/>
-      <c r="T61" s="209" t="n"/>
-      <c r="U61" s="209" t="n"/>
-      <c r="V61" s="209" t="n"/>
-      <c r="W61" s="209" t="n"/>
-      <c r="X61" s="209" t="n"/>
-      <c r="Y61" s="209" t="n"/>
-      <c r="Z61" s="209" t="n"/>
-      <c r="AA61" s="176" t="n"/>
-      <c r="AB61" s="176" t="n"/>
-      <c r="AC61" s="176" t="n"/>
-      <c r="AD61" s="176" t="n"/>
-      <c r="AE61" s="176" t="n"/>
-      <c r="AF61" s="176" t="n"/>
-      <c r="AG61" s="176" t="n"/>
-      <c r="AH61" s="176" t="n"/>
-      <c r="AI61" s="176" t="n"/>
-      <c r="AJ61" s="176" t="n"/>
-    </row>
-    <row r="62" ht="13.5" customHeight="1" s="122">
-      <c r="A62" s="123" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN62" s="123" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="9" customHeight="1" s="122"/>
-    <row r="64" ht="75" customHeight="1" s="122"/>
+    <row r="60" ht="9" customFormat="1" customHeight="1" s="176"/>
+    <row r="61" ht="75" customFormat="1" customHeight="1" s="176"/>
+    <row r="62" ht="13.5" customHeight="1" s="122"/>
+    <row r="63" ht="17.25" customHeight="1" s="122"/>
+    <row r="64" ht="17.25" customHeight="1" s="122"/>
     <row r="133" ht="17.25" customHeight="1" s="122"/>
     <row r="134" ht="17.25" customHeight="1" s="122"/>
     <row r="135" ht="17.25" customHeight="1" s="122"/>

</xml_diff>